<commit_message>
Update gas leads with sourced contacts, EPCs and revised close dates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdowns" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Named Contacts" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="ProjectStage">'Dropdowns'!$A$7:INDEX('Dropdowns'!$A$7:$A$106,COUNTA('Dropdowns'!$A$7:$A$106))</definedName>
@@ -1993,7 +1994,7 @@
         <v>48213</v>
       </c>
       <c r="X7" s="44" t="n">
-        <v>46843</v>
+        <v>47299</v>
       </c>
       <c r="Y7" s="45" t="n"/>
       <c r="Z7" s="37" t="inlineStr">
@@ -2048,12 +2049,12 @@
       </c>
       <c r="AJ7" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 2030 COD; public filings point to Dec 2031 (construction start Q4 2027). Cost not disclosed. Local opposition (water use). EPC not yet selected. Data-center tie not confirmed.</t>
+          <t>CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="AK7" s="38" t="inlineStr">
         <is>
-          <t>Contact Daniel Birmingham (Invenergy); track WI PSC CPCN filing for EPC selection; bundle with Union Depot CC.</t>
+          <t>Build relationship with Daniel Birmingham (Invenergy); watch PSC 5-CE-162 CPCN for EPC; get on EPC approved-vendor list in 2027.</t>
         </is>
       </c>
       <c r="AL7" s="38" t="inlineStr">
@@ -2115,7 +2116,7 @@
       </c>
       <c r="F8" s="36" t="inlineStr">
         <is>
-          <t>Eliecer Viamontes, President &amp; CEO</t>
+          <t>Keith Pollock, Project Director, OCAPS</t>
         </is>
       </c>
       <c r="G8" s="36" t="inlineStr">
@@ -2170,7 +2171,7 @@
         <v>46309</v>
       </c>
       <c r="X8" s="44" t="n">
-        <v>46387</v>
+        <v>46507</v>
       </c>
       <c r="Y8" s="45" t="n"/>
       <c r="Z8" s="37" t="inlineStr">
@@ -2225,12 +2226,12 @@
       </c>
       <c r="AJ8" s="38" t="inlineStr">
         <is>
-          <t>Plant is now operating; new-build cable window closed. Keep for MRO/aftermarket and relationship with TIC / Sargent &amp; Lundy for next Entergy builds. Yes Energy MW (1,306) differs from Entergy (1,215).</t>
+          <t>In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="AK8" s="38" t="inlineStr">
         <is>
-          <t>Reclassify as aftermarket/MRO; use TIC &amp; S&amp;L relationship for Entergy pipeline (Titanium, Waterford 5/6).</t>
+          <t>Aftermarket/spares with Keith Pollock and Entergy fossil ops supply chain; use TIC/S&amp;L relationship for Entergy program plants.</t>
         </is>
       </c>
       <c r="AL8" s="38" t="inlineStr">
@@ -2282,7 +2283,7 @@
       </c>
       <c r="F9" s="36" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Jim Burke, President &amp; CEO</t>
         </is>
       </c>
       <c r="G9" s="36" t="inlineStr">
@@ -2337,7 +2338,7 @@
         <v>46874</v>
       </c>
       <c r="X9" s="44" t="n">
-        <v>46477</v>
+        <v>46418</v>
       </c>
       <c r="Y9" s="45" t="n"/>
       <c r="Z9" s="37" t="inlineStr">
@@ -2392,12 +2393,12 @@
       </c>
       <c r="AJ9" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 2030; ERCOT/Cleanview show May 2028 COD. Link of ERCOT IDs to Vistra project based on GEM aliases + site/MW match. EPC and OEM not public. Urgent: procurement likely now-2027.</t>
+          <t>CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="AK9" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC via Vistra/TCEQ permit 178462; find Vistra Luminant project/procurement contact; quote both units (880 MW).</t>
+          <t>URGENT: identify EPC via TCEQ 178462 NAPD / Industrial Info; find Luminant project contact; quote both units (880 MW).</t>
         </is>
       </c>
       <c r="AL9" s="38" t="inlineStr">
@@ -2447,9 +2448,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>Rick Anderson, SVP &amp; Senior Production Officer</t>
         </is>
       </c>
       <c r="G10" s="36" t="inlineStr">
@@ -2460,7 +2461,7 @@
       <c r="H10" s="39" t="n"/>
       <c r="I10" s="37" t="inlineStr">
         <is>
-          <t>IOU</t>
+          <t>EPC</t>
         </is>
       </c>
       <c r="J10" s="40" t="n"/>
@@ -2504,7 +2505,7 @@
         <v>46568</v>
       </c>
       <c r="X10" s="44" t="n">
-        <v>46387</v>
+        <v>46371</v>
       </c>
       <c r="Y10" s="45" t="n"/>
       <c r="Z10" s="37" t="inlineStr">
@@ -2559,17 +2560,17 @@
       </c>
       <c r="AJ10" s="38" t="inlineStr">
         <is>
-          <t>Late stage - Unit 8 cable likely bought; Units 9/10 BOP and commissioning needs may still be open. Load growth driven largely by data centers (no named customer). EPC not public.</t>
+          <t>LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="AK10" s="38" t="inlineStr">
         <is>
-          <t>Confirm EPC/electrical contractor at Yates; position for Units 9-10 and Southern Co. future IRP gas units.</t>
+          <t>Relationship/spares play via B&amp;V site procurement; position with Mitsubishi/B&amp;V for next Georgia Power CT/CC builds.</t>
         </is>
       </c>
       <c r="AL10" s="38" t="inlineStr">
         <is>
-          <t>Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. Cost: Not public; PSC staff ~$1B for 3 units. EPC: Not public. OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE).</t>
+          <t>Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. Cost: Not public; PSC staff ~$1B for 3 units. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE).</t>
         </is>
       </c>
       <c r="AM10" s="40" t="n"/>
@@ -2614,9 +2615,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
-        <is>
-          <t>Laura Landreaux, President &amp; CEO</t>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz, VP, Power Development - New Generation</t>
         </is>
       </c>
       <c r="G11" s="36" t="inlineStr">
@@ -2627,7 +2628,7 @@
       <c r="H11" s="39" t="n"/>
       <c r="I11" s="37" t="inlineStr">
         <is>
-          <t>IOU</t>
+          <t>EPC</t>
         </is>
       </c>
       <c r="J11" s="40" t="n"/>
@@ -2668,7 +2669,7 @@
       </c>
       <c r="V11" s="40" t="n"/>
       <c r="W11" s="44" t="n">
-        <v>46935</v>
+        <v>47118</v>
       </c>
       <c r="X11" s="44" t="n">
         <v>46477</v>
@@ -2726,17 +2727,17 @@
       </c>
       <c r="AJ11" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 467.3 MW (EIA nameplate) and 2029; Entergy says 446 MW, late 2028. Vendor fair held Mar 2026 - subcontract procurement open; Entergy prioritizing Arkansas contractors. EPC not public (TIC possible).</t>
+          <t>CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="AK11" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC/GC (check TIC Entergy program); engage Arkansas electrical contractors from vendor fair.</t>
+          <t>Get on TSL Power Partners bidder list (Kiewit/TIC Lenexa) and S&amp;L approved-manufacturer list; register with Entergy supplier program.</t>
         </is>
       </c>
       <c r="AL11" s="38" t="inlineStr">
         <is>
-          <t>446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). Cost: Not disclosed (GAJA rider). EPC: Not public. OEM: Not found. Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). Cost: Not disclosed (GAJA rider). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM11" s="40" t="n"/>
@@ -2781,9 +2782,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
-        <is>
-          <t>Bill Norton, Spokesman</t>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>John Robert Smith Jr., General Manager, New Gas Generation Development</t>
         </is>
       </c>
       <c r="G12" s="38" t="inlineStr">
@@ -2835,10 +2836,10 @@
       </c>
       <c r="V12" s="40" t="n"/>
       <c r="W12" s="44" t="n">
-        <v>47119</v>
+        <v>47118</v>
       </c>
       <c r="X12" s="44" t="n">
-        <v>46477</v>
+        <v>46416</v>
       </c>
       <c r="Y12" s="45" t="n"/>
       <c r="Z12" s="37" t="inlineStr">
@@ -2893,12 +2894,12 @@
       </c>
       <c r="AJ12" s="38" t="inlineStr">
         <is>
-          <t>Utility is Duke Energy Progress (not DEC as in Yes Energy). CC1 COD ~late 2028/early 2029; 2030 is CC2. Microsoft bought nearby Person County Mega Park (supply tie not confirmed by Duke). BOP electrical peak 2027.</t>
+          <t>CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="AK12" s="38" t="inlineStr">
         <is>
-          <t>Engage Zachry procurement for CC1 + CC2 as one pursuit; ZIP 27343 to be confirmed.</t>
+          <t>Engage Zachry procurement now for CC1 (+CC2 combined buy); contact John Robert Smith Jr. (Duke PM&amp;C).</t>
         </is>
       </c>
       <c r="AL12" s="38" t="inlineStr">
@@ -2956,9 +2957,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
-        <is>
-          <t>Haley Fisackerly, President &amp; CEO</t>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>Ernest Rufus, Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
         </is>
       </c>
       <c r="G13" s="36" t="inlineStr">
@@ -3013,7 +3014,7 @@
         <v>46874</v>
       </c>
       <c r="X13" s="44" t="n">
-        <v>46387</v>
+        <v>46356</v>
       </c>
       <c r="Y13" s="45" t="n"/>
       <c r="Z13" s="37" t="inlineStr">
@@ -3068,12 +3069,12 @@
       </c>
       <c r="AJ13" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 879 MW / $651M; Entergy says 754 MW / $1.2B. Cable pulls likely 2026-early 2027 - window closing. Indirect tie to AWS Mississippi buildout.</t>
+          <t>MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="AK13" s="38" t="inlineStr">
         <is>
-          <t>Contact TSL Power Partners / Kiewit Power Constructors electrical procurement now; leverage for Vicksburg.</t>
+          <t>Contact Ernest Rufus and TSL/TIC procurement now - target program buy for Vicksburg/Ironwood/Waterford.</t>
         </is>
       </c>
       <c r="AL13" s="38" t="inlineStr">
@@ -3133,9 +3134,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>Haley Fisackerly, President &amp; CEO</t>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>Ernest Rufus, Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
         </is>
       </c>
       <c r="G14" s="36" t="inlineStr">
@@ -3146,7 +3147,7 @@
       <c r="H14" s="39" t="n"/>
       <c r="I14" s="37" t="inlineStr">
         <is>
-          <t>IOU</t>
+          <t>EPC</t>
         </is>
       </c>
       <c r="J14" s="40" t="n"/>
@@ -3190,7 +3191,7 @@
         <v>46966</v>
       </c>
       <c r="X14" s="44" t="n">
-        <v>46477</v>
+        <v>46371</v>
       </c>
       <c r="Y14" s="45" t="n"/>
       <c r="Z14" s="37" t="inlineStr">
@@ -3245,17 +3246,17 @@
       </c>
       <c r="AJ14" s="38" t="inlineStr">
         <is>
-          <t>Best-timed Mississippi lead - ~1 year behind Delta Blues; procurement now-2027. EPC and turbine OEM not confirmed. AWS link contextual, not dedicated.</t>
+          <t>URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="AK14" s="38" t="inlineStr">
         <is>
-          <t>Confirm EPC (check if TSL/Kiewit again) via MS PSC certificate / MDEQ air permit; position early.</t>
+          <t>Engage TSL/TIC procurement and Ernest Rufus immediately.</t>
         </is>
       </c>
       <c r="AL14" s="38" t="inlineStr">
         <is>
-          <t>754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. Cost: ~$1.2B (Entergy); Yes Energy $700M not confirmed. EPC: Not public. OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. Cost: ~$1.2B (Entergy); Yes Energy $700M not confirmed. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM14" s="40" t="n"/>
@@ -3300,9 +3301,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F15" s="36" t="inlineStr">
-        <is>
-          <t>Steve Baker, President &amp; COO</t>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>John E. Niland, VP, New Technology &amp; Thermal Development</t>
         </is>
       </c>
       <c r="G15" s="36" t="inlineStr">
@@ -3359,7 +3360,7 @@
         <v>47208</v>
       </c>
       <c r="X15" s="44" t="n">
-        <v>46660</v>
+        <v>46568</v>
       </c>
       <c r="Y15" s="45" t="n"/>
       <c r="Z15" s="37" t="inlineStr">
@@ -3414,17 +3415,17 @@
       </c>
       <c r="AJ15" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy record outdated: RTO is PJM (not MISO), 918 MW simple cycle (not 1,150 MW CC), COD 2029 (not 2027), not yet under construction. I&amp;M load growth driven by AWS/Google/Microsoft data centers. Do not confuse with Maple Creek Energy (same county).</t>
+          <t>CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="AK15" s="38" t="inlineStr">
         <is>
-          <t>Engage Invenergy Thermal now (EPC not awarded/public); track IURC Cause 46389 final order.</t>
+          <t>Engage Boldt procurement and Invenergy thermal construction now (Q4 2026-Q1 2027) for MV/600V/tray bid lists.</t>
         </is>
       </c>
       <c r="AL15" s="38" t="inlineStr">
         <is>
-          <t>~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. Cost: ~$500M capital investment (Invenergy). EPC: Not public. OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM).</t>
+          <t>~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. Cost: ~$500M capital investment (Invenergy). EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM).</t>
         </is>
       </c>
       <c r="AM15" s="40" t="n"/>
@@ -3469,9 +3470,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F16" s="36" t="inlineStr">
-        <is>
-          <t>Phillip May, President &amp; CEO</t>
+      <c r="F16" s="38" t="inlineStr">
+        <is>
+          <t>Nicholas D. Pressler, Director, Power Development</t>
         </is>
       </c>
       <c r="G16" s="38" t="inlineStr">
@@ -3528,7 +3529,7 @@
         <v>47088</v>
       </c>
       <c r="X16" s="44" t="n">
-        <v>46477</v>
+        <v>46416</v>
       </c>
       <c r="Y16" s="45" t="n"/>
       <c r="Z16" s="37" t="inlineStr">
@@ -3583,12 +3584,12 @@
       </c>
       <c r="AJ16" s="38" t="inlineStr">
         <is>
-          <t>COD late 2028 (2030 in Yes Energy is Hyperion full operation). Related ~100 mi 500 kV transmission program (~$1.2B) is a separate opportunity; ~7 more Hyperion plants (5.2 GW) up for LPSC vote Dec 2026.</t>
+          <t>CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="AK16" s="38" t="inlineStr">
         <is>
-          <t>Engage TIC / TSL Power Partners procurement; open separate opportunity for Entergy 500 kV transmission lines.</t>
+          <t>Engage TSL/TIC procurement now; contact Nicholas Pressler; open separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="AL16" s="38" t="inlineStr">
@@ -3638,9 +3639,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="F17" s="36" t="inlineStr">
-        <is>
-          <t>Phillip May, President &amp; CEO</t>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>Nicholas D. Pressler, Director, Power Development</t>
         </is>
       </c>
       <c r="G17" s="36" t="inlineStr">
@@ -3697,7 +3698,7 @@
         <v>47270</v>
       </c>
       <c r="X17" s="44" t="n">
-        <v>46568</v>
+        <v>46660</v>
       </c>
       <c r="Y17" s="45" t="n"/>
       <c r="Z17" s="37" t="inlineStr">
@@ -3752,17 +3753,17 @@
       </c>
       <c r="AJ17" s="38" t="inlineStr">
         <is>
-          <t>Waterford 6 (754 MW, ~Jul 2030) uses the same EPC - follow-on opportunity. MW varies by source (750-820). EPC name not yet public (possibly TIC/S&amp;L team).</t>
+          <t>CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="AK17" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC from LPSC Waterford 6 filing; pursue Waterford 5 + 6 together.</t>
+          <t>Pitch combined Waterford 5+6 cable package to TSL; contact Nicholas Pressler.</t>
         </is>
       </c>
       <c r="AL17" s="38" t="inlineStr">
         <is>
-          <t>1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. Cost: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. EPC: Not public. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. Cost: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM17" s="40" t="n"/>
@@ -14836,12 +14837,12 @@
       <c r="CF7" s="39" t="n"/>
       <c r="CG7" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 2030 COD; public filings point to Dec 2031 (construction start Q4 2027). Cost not disclosed. Local opposition (water use). EPC not yet selected. Data-center tie not confirmed.</t>
+          <t>CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="CH7" s="38" t="inlineStr">
         <is>
-          <t>Contact Daniel Birmingham (Invenergy); track WI PSC CPCN filing for EPC selection; bundle with Union Depot CC.</t>
+          <t>Build relationship with Daniel Birmingham (Invenergy); watch PSC 5-CE-162 CPCN for EPC; get on EPC approved-vendor list in 2027.</t>
         </is>
       </c>
       <c r="CI7" s="38" t="inlineStr">
@@ -14858,12 +14859,12 @@
     <row r="8" ht="23" customHeight="1">
       <c r="A8" s="36" t="inlineStr">
         <is>
-          <t>Viamontes</t>
+          <t>Pollock</t>
         </is>
       </c>
       <c r="B8" s="36" t="inlineStr">
         <is>
-          <t>Eliecer</t>
+          <t>Keith</t>
         </is>
       </c>
       <c r="C8" s="36" t="inlineStr">
@@ -14889,7 +14890,7 @@
       <c r="G8" s="40" t="n"/>
       <c r="H8" s="36" t="inlineStr">
         <is>
-          <t>President &amp; CEO</t>
+          <t>Project Director, OCAPS</t>
         </is>
       </c>
       <c r="I8" s="37" t="inlineStr">
@@ -15126,12 +15127,12 @@
       <c r="CF8" s="39" t="n"/>
       <c r="CG8" s="38" t="inlineStr">
         <is>
-          <t>Plant is now operating; new-build cable window closed. Keep for MRO/aftermarket and relationship with TIC / Sargent &amp; Lundy for next Entergy builds. Yes Energy MW (1,306) differs from Entergy (1,215).</t>
+          <t>In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="CH8" s="38" t="inlineStr">
         <is>
-          <t>Reclassify as aftermarket/MRO; use TIC &amp; S&amp;L relationship for Entergy pipeline (Titanium, Waterford 5/6).</t>
+          <t>Aftermarket/spares with Keith Pollock and Entergy fossil ops supply chain; use TIC/S&amp;L relationship for Entergy program plants.</t>
         </is>
       </c>
       <c r="CI8" s="38" t="inlineStr">
@@ -15148,13 +15149,17 @@
     <row r="9" ht="23" customHeight="1">
       <c r="A9" s="36" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="B9" s="39" t="n"/>
+          <t>Burke</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>Jim</t>
+        </is>
+      </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Vistra Corp (Luminant)</t>
+          <t>Vistra Corp</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -15175,7 +15180,7 @@
       <c r="G9" s="40" t="n"/>
       <c r="H9" s="36" t="inlineStr">
         <is>
-          <t>Project / Procurement contact</t>
+          <t>President &amp; CEO</t>
         </is>
       </c>
       <c r="I9" s="37" t="inlineStr">
@@ -15408,12 +15413,12 @@
       <c r="CF9" s="39" t="n"/>
       <c r="CG9" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 2030; ERCOT/Cleanview show May 2028 COD. Link of ERCOT IDs to Vistra project based on GEM aliases + site/MW match. EPC and OEM not public. Urgent: procurement likely now-2027.</t>
+          <t>CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="CH9" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC via Vistra/TCEQ permit 178462; find Vistra Luminant project/procurement contact; quote both units (880 MW).</t>
+          <t>URGENT: identify EPC via TCEQ 178462 NAPD / Industrial Info; find Luminant project contact; quote both units (880 MW).</t>
         </is>
       </c>
       <c r="CI9" s="38" t="inlineStr">
@@ -15430,10 +15435,14 @@
     <row r="10" ht="23" customHeight="1">
       <c r="A10" s="36" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="B10" s="39" t="n"/>
+          <t>Anderson</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>Rick</t>
+        </is>
+      </c>
       <c r="C10" s="36" t="inlineStr">
         <is>
           <t>Georgia Power</t>
@@ -15457,7 +15466,7 @@
       <c r="G10" s="40" t="n"/>
       <c r="H10" s="36" t="inlineStr">
         <is>
-          <t>Project / Procurement contact</t>
+          <t>SVP &amp; Senior Production Officer</t>
         </is>
       </c>
       <c r="I10" s="37" t="inlineStr">
@@ -15613,7 +15622,11 @@
           <t>Georgia Power</t>
         </is>
       </c>
-      <c r="BF10" s="39" t="n"/>
+      <c r="BF10" s="38" t="inlineStr">
+        <is>
+          <t>Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024)</t>
+        </is>
+      </c>
       <c r="BG10" s="36" t="inlineStr">
         <is>
           <t>Georgia Power</t>
@@ -15694,12 +15707,12 @@
       <c r="CF10" s="39" t="n"/>
       <c r="CG10" s="38" t="inlineStr">
         <is>
-          <t>Late stage - Unit 8 cable likely bought; Units 9/10 BOP and commissioning needs may still be open. Load growth driven largely by data centers (no named customer). EPC not public.</t>
+          <t>LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="CH10" s="38" t="inlineStr">
         <is>
-          <t>Confirm EPC/electrical contractor at Yates; position for Units 9-10 and Southern Co. future IRP gas units.</t>
+          <t>Relationship/spares play via B&amp;V site procurement; position with Mitsubishi/B&amp;V for next Georgia Power CT/CC builds.</t>
         </is>
       </c>
       <c r="CI10" s="38" t="inlineStr">
@@ -15716,17 +15729,17 @@
     <row r="11" ht="23" customHeight="1">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>Landreaux</t>
+          <t>Ruiz</t>
         </is>
       </c>
       <c r="B11" s="36" t="inlineStr">
         <is>
-          <t>Laura</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Entergy Arkansas</t>
+          <t>Entergy</t>
         </is>
       </c>
       <c r="D11" s="37" t="inlineStr">
@@ -15747,7 +15760,7 @@
       <c r="G11" s="40" t="n"/>
       <c r="H11" s="36" t="inlineStr">
         <is>
-          <t>President &amp; CEO</t>
+          <t>VP, Power Development - New Generation</t>
         </is>
       </c>
       <c r="I11" s="37" t="inlineStr">
@@ -15811,7 +15824,7 @@
       <c r="AI11" s="41" t="n"/>
       <c r="AJ11" s="49" t="n"/>
       <c r="AK11" s="44" t="n">
-        <v>46935</v>
+        <v>47118</v>
       </c>
       <c r="AL11" s="43" t="n">
         <v>446</v>
@@ -15899,14 +15912,22 @@
           <t>Entergy Arkansas</t>
         </is>
       </c>
-      <c r="BF11" s="39" t="n"/>
+      <c r="BF11" s="38" t="inlineStr">
+        <is>
+          <t>TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page)</t>
+        </is>
+      </c>
       <c r="BG11" s="36" t="inlineStr">
         <is>
           <t>Entergy Arkansas</t>
         </is>
       </c>
       <c r="BH11" s="39" t="n"/>
-      <c r="BI11" s="39" t="n"/>
+      <c r="BI11" s="38" t="inlineStr">
+        <is>
+          <t>Mitsubishi Power (implied by TSL/MPWA program)</t>
+        </is>
+      </c>
       <c r="BJ11" s="39" t="n"/>
       <c r="BK11" s="39" t="n"/>
       <c r="BL11" s="38" t="inlineStr">
@@ -15976,12 +15997,12 @@
       <c r="CF11" s="39" t="n"/>
       <c r="CG11" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 467.3 MW (EIA nameplate) and 2029; Entergy says 446 MW, late 2028. Vendor fair held Mar 2026 - subcontract procurement open; Entergy prioritizing Arkansas contractors. EPC not public (TIC possible).</t>
+          <t>CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="CH11" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC/GC (check TIC Entergy program); engage Arkansas electrical contractors from vendor fair.</t>
+          <t>Get on TSL Power Partners bidder list (Kiewit/TIC Lenexa) and S&amp;L approved-manufacturer list; register with Entergy supplier program.</t>
         </is>
       </c>
       <c r="CI11" s="38" t="inlineStr">
@@ -15998,12 +16019,12 @@
     <row r="12" ht="23" customHeight="1">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Smith Jr.</t>
         </is>
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>Bill</t>
+          <t>John Robert</t>
         </is>
       </c>
       <c r="C12" s="36" t="inlineStr">
@@ -16027,9 +16048,9 @@
         </is>
       </c>
       <c r="G12" s="40" t="n"/>
-      <c r="H12" s="36" t="inlineStr">
-        <is>
-          <t>Spokesman</t>
+      <c r="H12" s="38" t="inlineStr">
+        <is>
+          <t>General Manager, New Gas Generation Development</t>
         </is>
       </c>
       <c r="I12" s="37" t="inlineStr">
@@ -16093,7 +16114,7 @@
       <c r="AI12" s="41" t="n"/>
       <c r="AJ12" s="49" t="n"/>
       <c r="AK12" s="44" t="n">
-        <v>47119</v>
+        <v>47118</v>
       </c>
       <c r="AL12" s="43" t="n">
         <v>1360</v>
@@ -16278,12 +16299,12 @@
       <c r="CF12" s="39" t="n"/>
       <c r="CG12" s="38" t="inlineStr">
         <is>
-          <t>Utility is Duke Energy Progress (not DEC as in Yes Energy). CC1 COD ~late 2028/early 2029; 2030 is CC2. Microsoft bought nearby Person County Mega Park (supply tie not confirmed by Duke). BOP electrical peak 2027.</t>
+          <t>CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="CH12" s="38" t="inlineStr">
         <is>
-          <t>Engage Zachry procurement for CC1 + CC2 as one pursuit; ZIP 27343 to be confirmed.</t>
+          <t>Engage Zachry procurement now for CC1 (+CC2 combined buy); contact John Robert Smith Jr. (Duke PM&amp;C).</t>
         </is>
       </c>
       <c r="CI12" s="38" t="inlineStr">
@@ -16300,17 +16321,17 @@
     <row r="13" ht="23" customHeight="1">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>Fisackerly</t>
+          <t>Rufus</t>
         </is>
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>Haley</t>
+          <t>Ernest</t>
         </is>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
-          <t>Entergy Mississippi</t>
+          <t>Entergy</t>
         </is>
       </c>
       <c r="D13" s="37" t="inlineStr">
@@ -16329,9 +16350,9 @@
         </is>
       </c>
       <c r="G13" s="40" t="n"/>
-      <c r="H13" s="36" t="inlineStr">
-        <is>
-          <t>President &amp; CEO</t>
+      <c r="H13" s="38" t="inlineStr">
+        <is>
+          <t>Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
         </is>
       </c>
       <c r="I13" s="37" t="inlineStr">
@@ -16582,12 +16603,12 @@
       <c r="CF13" s="39" t="n"/>
       <c r="CG13" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy shows 879 MW / $651M; Entergy says 754 MW / $1.2B. Cable pulls likely 2026-early 2027 - window closing. Indirect tie to AWS Mississippi buildout.</t>
+          <t>MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="CH13" s="38" t="inlineStr">
         <is>
-          <t>Contact TSL Power Partners / Kiewit Power Constructors electrical procurement now; leverage for Vicksburg.</t>
+          <t>Contact Ernest Rufus and TSL/TIC procurement now - target program buy for Vicksburg/Ironwood/Waterford.</t>
         </is>
       </c>
       <c r="CI13" s="38" t="inlineStr">
@@ -16604,17 +16625,17 @@
     <row r="14" ht="23" customHeight="1">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>Fisackerly</t>
+          <t>Rufus</t>
         </is>
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>Haley</t>
+          <t>Ernest</t>
         </is>
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Entergy Mississippi</t>
+          <t>Entergy</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
@@ -16633,9 +16654,9 @@
         </is>
       </c>
       <c r="G14" s="40" t="n"/>
-      <c r="H14" s="36" t="inlineStr">
-        <is>
-          <t>President &amp; CEO</t>
+      <c r="H14" s="38" t="inlineStr">
+        <is>
+          <t>Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
         </is>
       </c>
       <c r="I14" s="37" t="inlineStr">
@@ -16757,7 +16778,7 @@
       </c>
       <c r="AX14" s="38" t="inlineStr">
         <is>
-          <t>Former Baxter Wilson Steam Electric Station site</t>
+          <t>770 Kemp Bottom Rd (former Baxter Wilson site)</t>
         </is>
       </c>
       <c r="AY14" s="36" t="inlineStr">
@@ -16787,7 +16808,11 @@
           <t>Entergy Mississippi</t>
         </is>
       </c>
-      <c r="BF14" s="39" t="n"/>
+      <c r="BF14" s="38" t="inlineStr">
+        <is>
+          <t>TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page)</t>
+        </is>
+      </c>
       <c r="BG14" s="36" t="inlineStr">
         <is>
           <t>Entergy Mississippi</t>
@@ -16868,12 +16893,12 @@
       <c r="CF14" s="39" t="n"/>
       <c r="CG14" s="38" t="inlineStr">
         <is>
-          <t>Best-timed Mississippi lead - ~1 year behind Delta Blues; procurement now-2027. EPC and turbine OEM not confirmed. AWS link contextual, not dedicated.</t>
+          <t>URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="CH14" s="38" t="inlineStr">
         <is>
-          <t>Confirm EPC (check if TSL/Kiewit again) via MS PSC certificate / MDEQ air permit; position early.</t>
+          <t>Engage TSL/TIC procurement and Ernest Rufus immediately.</t>
         </is>
       </c>
       <c r="CI14" s="38" t="inlineStr">
@@ -16890,17 +16915,17 @@
     <row r="15" ht="23" customHeight="1">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Baker</t>
+          <t>Niland</t>
         </is>
       </c>
       <c r="B15" s="36" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>John E.</t>
         </is>
       </c>
       <c r="C15" s="36" t="inlineStr">
         <is>
-          <t>Indiana Michigan Power (AEP)</t>
+          <t>Invenergy</t>
         </is>
       </c>
       <c r="D15" s="37" t="inlineStr">
@@ -16921,12 +16946,12 @@
       <c r="G15" s="40" t="n"/>
       <c r="H15" s="36" t="inlineStr">
         <is>
-          <t>President &amp; COO</t>
+          <t>VP, New Technology &amp; Thermal Development</t>
         </is>
       </c>
       <c r="I15" s="37" t="inlineStr">
         <is>
-          <t>End User</t>
+          <t>Contractor</t>
         </is>
       </c>
       <c r="J15" s="37" t="inlineStr">
@@ -17075,7 +17100,11 @@
           <t>Invenergy (to be acquired by I&amp;M at COD)</t>
         </is>
       </c>
-      <c r="BF15" s="39" t="n"/>
+      <c r="BF15" s="38" t="inlineStr">
+        <is>
+          <t>The Boldt Company (constructor per Boldt project page - role to confirm)</t>
+        </is>
+      </c>
       <c r="BG15" s="36" t="inlineStr">
         <is>
           <t>Invenergy</t>
@@ -17156,12 +17185,12 @@
       <c r="CF15" s="39" t="n"/>
       <c r="CG15" s="38" t="inlineStr">
         <is>
-          <t>Yes Energy record outdated: RTO is PJM (not MISO), 918 MW simple cycle (not 1,150 MW CC), COD 2029 (not 2027), not yet under construction. I&amp;M load growth driven by AWS/Google/Microsoft data centers. Do not confuse with Maple Creek Energy (same county).</t>
+          <t>CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="CH15" s="38" t="inlineStr">
         <is>
-          <t>Engage Invenergy Thermal now (EPC not awarded/public); track IURC Cause 46389 final order.</t>
+          <t>Engage Boldt procurement and Invenergy thermal construction now (Q4 2026-Q1 2027) for MV/600V/tray bid lists.</t>
         </is>
       </c>
       <c r="CI15" s="38" t="inlineStr">
@@ -17178,17 +17207,17 @@
     <row r="16" ht="23" customHeight="1">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Pressler</t>
         </is>
       </c>
       <c r="B16" s="36" t="inlineStr">
         <is>
-          <t>Phillip</t>
+          <t>Nicholas D.</t>
         </is>
       </c>
       <c r="C16" s="36" t="inlineStr">
         <is>
-          <t>Entergy Louisiana</t>
+          <t>Entergy Services LLC</t>
         </is>
       </c>
       <c r="D16" s="37" t="inlineStr">
@@ -17209,7 +17238,7 @@
       <c r="G16" s="40" t="n"/>
       <c r="H16" s="36" t="inlineStr">
         <is>
-          <t>President &amp; CEO</t>
+          <t>Director, Power Development</t>
         </is>
       </c>
       <c r="I16" s="37" t="inlineStr">
@@ -17448,12 +17477,12 @@
       <c r="CF16" s="39" t="n"/>
       <c r="CG16" s="38" t="inlineStr">
         <is>
-          <t>COD late 2028 (2030 in Yes Energy is Hyperion full operation). Related ~100 mi 500 kV transmission program (~$1.2B) is a separate opportunity; ~7 more Hyperion plants (5.2 GW) up for LPSC vote Dec 2026.</t>
+          <t>CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="CH16" s="38" t="inlineStr">
         <is>
-          <t>Engage TIC / TSL Power Partners procurement; open separate opportunity for Entergy 500 kV transmission lines.</t>
+          <t>Engage TSL/TIC procurement now; contact Nicholas Pressler; open separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="CI16" s="38" t="inlineStr">
@@ -17470,17 +17499,17 @@
     <row r="17" ht="23" customHeight="1">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Pressler</t>
         </is>
       </c>
       <c r="B17" s="36" t="inlineStr">
         <is>
-          <t>Phillip</t>
+          <t>Nicholas D.</t>
         </is>
       </c>
       <c r="C17" s="36" t="inlineStr">
         <is>
-          <t>Entergy Louisiana</t>
+          <t>Entergy Services LLC</t>
         </is>
       </c>
       <c r="D17" s="37" t="inlineStr">
@@ -17501,7 +17530,7 @@
       <c r="G17" s="40" t="n"/>
       <c r="H17" s="36" t="inlineStr">
         <is>
-          <t>President &amp; CEO</t>
+          <t>Director, Power Development</t>
         </is>
       </c>
       <c r="I17" s="37" t="inlineStr">
@@ -17655,7 +17684,11 @@
           <t>Entergy Louisiana</t>
         </is>
       </c>
-      <c r="BF17" s="39" t="n"/>
+      <c r="BF17" s="38" t="inlineStr">
+        <is>
+          <t>TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing</t>
+        </is>
+      </c>
       <c r="BG17" s="36" t="inlineStr">
         <is>
           <t>Entergy Louisiana</t>
@@ -17746,12 +17779,12 @@
       <c r="CF17" s="39" t="n"/>
       <c r="CG17" s="38" t="inlineStr">
         <is>
-          <t>Waterford 6 (754 MW, ~Jul 2030) uses the same EPC - follow-on opportunity. MW varies by source (750-820). EPC name not yet public (possibly TIC/S&amp;L team).</t>
+          <t>CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="CH17" s="38" t="inlineStr">
         <is>
-          <t>Identify EPC from LPSC Waterford 6 filing; pursue Waterford 5 + 6 together.</t>
+          <t>Pitch combined Waterford 5+6 cable package to TSL; contact Nicholas Pressler.</t>
         </is>
       </c>
       <c r="CI17" s="38" t="inlineStr">
@@ -44417,4 +44450,1538 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="52" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B1" s="52" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="52" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="52" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="E1" s="52" t="inlineStr">
+        <is>
+          <t>Role on project</t>
+        </is>
+      </c>
+      <c r="F1" s="52" t="inlineStr">
+        <is>
+          <t>Published business contact</t>
+        </is>
+      </c>
+      <c r="G1" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="H1" s="52" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B2" s="53" t="inlineStr">
+        <is>
+          <t>Daniel Birmingham</t>
+        </is>
+      </c>
+      <c r="C2" s="53" t="inlineStr">
+        <is>
+          <t>Lead Developer</t>
+        </is>
+      </c>
+      <c r="D2" s="53" t="inlineStr">
+        <is>
+          <t>Invenergy</t>
+        </is>
+      </c>
+      <c r="E2" s="53" t="inlineStr">
+        <is>
+          <t>Developer lead</t>
+        </is>
+      </c>
+      <c r="F2" s="53" t="inlineStr"/>
+      <c r="G2" s="53" t="inlineStr">
+        <is>
+          <t>https://www.nbc26.com/lakeshore/two-natural-gas-power-plants-proposed-in-brillion</t>
+        </is>
+      </c>
+      <c r="H2" s="53" t="inlineStr">
+        <is>
+          <t>News quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B3" s="53" t="inlineStr">
+        <is>
+          <t>Brendan Conway</t>
+        </is>
+      </c>
+      <c r="C3" s="53" t="inlineStr">
+        <is>
+          <t>Spokesperson</t>
+        </is>
+      </c>
+      <c r="D3" s="53" t="inlineStr">
+        <is>
+          <t>We Energies</t>
+        </is>
+      </c>
+      <c r="E3" s="53" t="inlineStr">
+        <is>
+          <t>Possible acquirer</t>
+        </is>
+      </c>
+      <c r="F3" s="53" t="inlineStr"/>
+      <c r="G3" s="53" t="inlineStr">
+        <is>
+          <t>https://www.wpr.org/news/energy-developer-planning-2-gigawatt-natural-gas-plants-northeast-wisconsin</t>
+        </is>
+      </c>
+      <c r="H3" s="53" t="inlineStr">
+        <is>
+          <t>News quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="53" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B4" s="53" t="inlineStr">
+        <is>
+          <t>Keith Pollock</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>Project Director, OCAPS</t>
+        </is>
+      </c>
+      <c r="D4" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Texas</t>
+        </is>
+      </c>
+      <c r="E4" s="53" t="inlineStr">
+        <is>
+          <t>Owner project lead</t>
+        </is>
+      </c>
+      <c r="F4" s="53" t="inlineStr"/>
+      <c r="G4" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/construction-nears-completion-on-entergy-texas-orange-county-advanced-power-station</t>
+        </is>
+      </c>
+      <c r="H4" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>David Borde</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Texas</t>
+        </is>
+      </c>
+      <c r="E5" s="53" t="inlineStr">
+        <is>
+          <t>Executive</t>
+        </is>
+      </c>
+      <c r="F5" s="53" t="inlineStr"/>
+      <c r="G5" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-texas-orange-county-advanced-power-station-begins-delivering-reliable-power-to-southeast-texas</t>
+        </is>
+      </c>
+      <c r="H5" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="53" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="inlineStr">
+        <is>
+          <t>James Malone</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="inlineStr">
+        <is>
+          <t>Director of Business Development</t>
+        </is>
+      </c>
+      <c r="D6" s="53" t="inlineStr">
+        <is>
+          <t>Sargent &amp; Lundy</t>
+        </is>
+      </c>
+      <c r="E6" s="53" t="inlineStr">
+        <is>
+          <t>Engineer of record</t>
+        </is>
+      </c>
+      <c r="F6" s="53" t="inlineStr"/>
+      <c r="G6" s="53" t="inlineStr">
+        <is>
+          <t>https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+        </is>
+      </c>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>Company website</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="inlineStr">
+        <is>
+          <t>Kendra James</t>
+        </is>
+      </c>
+      <c r="C7" s="53" t="inlineStr">
+        <is>
+          <t>Media Relations</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Texas</t>
+        </is>
+      </c>
+      <c r="E7" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F7" s="53" t="inlineStr">
+        <is>
+          <t>Media line 281-297-2353</t>
+        </is>
+      </c>
+      <c r="G7" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/media-kit</t>
+        </is>
+      </c>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>Jim Burke</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr">
+        <is>
+          <t>Vistra Corp</t>
+        </is>
+      </c>
+      <c r="E8" s="53" t="inlineStr">
+        <is>
+          <t>Executive (no project contact public)</t>
+        </is>
+      </c>
+      <c r="F8" s="53" t="inlineStr"/>
+      <c r="G8" s="53" t="inlineStr">
+        <is>
+          <t>https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas</t>
+        </is>
+      </c>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B9" s="53" t="inlineStr">
+        <is>
+          <t>Rick Anderson</t>
+        </is>
+      </c>
+      <c r="C9" s="53" t="inlineStr">
+        <is>
+          <t>SVP &amp; Senior Production Officer</t>
+        </is>
+      </c>
+      <c r="D9" s="53" t="inlineStr">
+        <is>
+          <t>Georgia Power</t>
+        </is>
+      </c>
+      <c r="E9" s="53" t="inlineStr">
+        <is>
+          <t>Owner executive</t>
+        </is>
+      </c>
+      <c r="F9" s="53" t="inlineStr"/>
+      <c r="G9" s="53" t="inlineStr">
+        <is>
+          <t>https://www.georgiapower.com/news-hub/press-releases/first-new-natural-gas-turbine-delivered-to-georgia-power-plant-yates.html</t>
+        </is>
+      </c>
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="53" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B10" s="53" t="inlineStr">
+        <is>
+          <t>Cheryl Boddiford</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="inlineStr">
+        <is>
+          <t>SVP, North American Manufacturing &amp; Supply Chain Mgmt</t>
+        </is>
+      </c>
+      <c r="D10" s="53" t="inlineStr">
+        <is>
+          <t>Mitsubishi Power</t>
+        </is>
+      </c>
+      <c r="E10" s="53" t="inlineStr">
+        <is>
+          <t>EPC consortium (OEM)</t>
+        </is>
+      </c>
+      <c r="F10" s="53" t="inlineStr"/>
+      <c r="G10" s="53" t="inlineStr">
+        <is>
+          <t>https://power.mhi.com/regions/amer/news/250819</t>
+        </is>
+      </c>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="53" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B11" s="53" t="inlineStr">
+        <is>
+          <t>Rick Janik</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>Project Manager (Plant Barry Unit 8)</t>
+        </is>
+      </c>
+      <c r="D11" s="53" t="inlineStr">
+        <is>
+          <t>Black &amp; Veatch</t>
+        </is>
+      </c>
+      <c r="E11" s="53" t="inlineStr">
+        <is>
+          <t>Same EPC pairing at Southern Co. - not confirmed for Yates</t>
+        </is>
+      </c>
+      <c r="F11" s="53" t="inlineStr"/>
+      <c r="G11" s="53" t="inlineStr">
+        <is>
+          <t>https://www.bv.com/en-US/projects/gas-fired-power-plant-project-defies-challenges-to-deliver-safe-reliable-power</t>
+        </is>
+      </c>
+      <c r="H11" s="53" t="inlineStr">
+        <is>
+          <t>Company website - indirect</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="inlineStr">
+        <is>
+          <t>VP, Power Development - New Generation</t>
+        </is>
+      </c>
+      <c r="D12" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E12" s="53" t="inlineStr">
+        <is>
+          <t>Owner new-generation executive</t>
+        </is>
+      </c>
+      <c r="F12" s="53" t="inlineStr"/>
+      <c r="G12" s="53" t="inlineStr">
+        <is>
+          <t>https://apps.apsc.arkansas.gov/pdf/24/24-072-U_67_1.pdf</t>
+        </is>
+      </c>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="inlineStr">
+        <is>
+          <t>Laura Landreaux</t>
+        </is>
+      </c>
+      <c r="C13" s="53" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D13" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Arkansas</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>Executive</t>
+        </is>
+      </c>
+      <c r="F13" s="53" t="inlineStr"/>
+      <c r="G13" s="53" t="inlineStr">
+        <is>
+          <t>https://www.arkansasonline.com/news/2026/aug/21/entergy-breaks-ground-on-ironwood-power-station/</t>
+        </is>
+      </c>
+      <c r="H13" s="53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B14" s="53" t="inlineStr">
+        <is>
+          <t>Louise Duncan</t>
+        </is>
+      </c>
+      <c r="C14" s="53" t="inlineStr">
+        <is>
+          <t>VP, Power Plant Operations</t>
+        </is>
+      </c>
+      <c r="D14" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Arkansas</t>
+        </is>
+      </c>
+      <c r="E14" s="53" t="inlineStr">
+        <is>
+          <t>Plant operations</t>
+        </is>
+      </c>
+      <c r="F14" s="53" t="inlineStr"/>
+      <c r="G14" s="53" t="inlineStr">
+        <is>
+          <t>https://adeq.state.ar.us/downloads/WebDatabases/PermitsOnline/NPDES/PermitInformation/AR0001147_Certificate%20of%20Service%20Letter_20260430.pdf</t>
+        </is>
+      </c>
+      <c r="H14" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory document</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B15" s="53" t="inlineStr">
+        <is>
+          <t>Clay McMaster</t>
+        </is>
+      </c>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t>Environmental/permit contact, Lake Catherine</t>
+        </is>
+      </c>
+      <c r="D15" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E15" s="53" t="inlineStr">
+        <is>
+          <t>Permitting</t>
+        </is>
+      </c>
+      <c r="F15" s="53" t="inlineStr">
+        <is>
+          <t>wmcmast@entergy.com (ADEQ permit)</t>
+        </is>
+      </c>
+      <c r="G15" s="53" t="inlineStr">
+        <is>
+          <t>https://adeq.state.ar.us/downloads/WebDatabases/PermitsOnline/Air/1717-AOP-R9.pdf</t>
+        </is>
+      </c>
+      <c r="H15" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory document</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B16" s="53" t="inlineStr">
+        <is>
+          <t>Kendall Thornton</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="inlineStr">
+        <is>
+          <t>Stakeholder Engagement Coordinator</t>
+        </is>
+      </c>
+      <c r="D16" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Arkansas</t>
+        </is>
+      </c>
+      <c r="E16" s="53" t="inlineStr">
+        <is>
+          <t>Groundbreaking organizer</t>
+        </is>
+      </c>
+      <c r="F16" s="53" t="inlineStr"/>
+      <c r="G16" s="53" t="inlineStr">
+        <is>
+          <t>https://arkansasstatechamber.com/team-member/kendall-thornton/</t>
+        </is>
+      </c>
+      <c r="H16" s="53" t="inlineStr">
+        <is>
+          <t>Org website</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="inlineStr">
+        <is>
+          <t>Jason Rees</t>
+        </is>
+      </c>
+      <c r="C17" s="53" t="inlineStr">
+        <is>
+          <t>Director of Procurement</t>
+        </is>
+      </c>
+      <c r="D17" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E17" s="53" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="F17" s="53" t="inlineStr"/>
+      <c r="G17" s="53" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/reesjason/</t>
+        </is>
+      </c>
+      <c r="H17" s="53" t="inlineStr">
+        <is>
+          <t>LinkedIn - verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="53" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B18" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Supplier Registration</t>
+        </is>
+      </c>
+      <c r="C18" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E18" s="53" t="inlineStr">
+        <is>
+          <t>Supplier onboarding</t>
+        </is>
+      </c>
+      <c r="F18" s="53" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com; 844-387-9675</t>
+        </is>
+      </c>
+      <c r="G18" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/suppliers/how</t>
+        </is>
+      </c>
+      <c r="H18" s="53" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="53" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B19" s="53" t="inlineStr">
+        <is>
+          <t>John Robert Smith Jr.</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="inlineStr">
+        <is>
+          <t>GM, New Gas Generation Development (PM&amp;C)</t>
+        </is>
+      </c>
+      <c r="D19" s="53" t="inlineStr">
+        <is>
+          <t>Duke Energy</t>
+        </is>
+      </c>
+      <c r="E19" s="53" t="inlineStr">
+        <is>
+          <t>Owner project development lead</t>
+        </is>
+      </c>
+      <c r="F19" s="53" t="inlineStr"/>
+      <c r="G19" s="53" t="inlineStr">
+        <is>
+          <t>https://starw1.ncuc.gov/NCUC/ViewFile.aspx?Id=5552fef5-9b1f-4e88-b9ca-0e649dafdbb5</t>
+        </is>
+      </c>
+      <c r="H19" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="53" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>Ralph Biediger</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>EPC Group President</t>
+        </is>
+      </c>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>Zachry Group</t>
+        </is>
+      </c>
+      <c r="E20" s="53" t="inlineStr">
+        <is>
+          <t>EPC executive</t>
+        </is>
+      </c>
+      <c r="F20" s="53" t="inlineStr"/>
+      <c r="G20" s="53" t="inlineStr">
+        <is>
+          <t>https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html</t>
+        </is>
+      </c>
+      <c r="H20" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="53" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B21" s="53" t="inlineStr">
+        <is>
+          <t>Bill Norton</t>
+        </is>
+      </c>
+      <c r="C21" s="53" t="inlineStr">
+        <is>
+          <t>Spokesperson</t>
+        </is>
+      </c>
+      <c r="D21" s="53" t="inlineStr">
+        <is>
+          <t>Duke Energy</t>
+        </is>
+      </c>
+      <c r="E21" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F21" s="53" t="inlineStr"/>
+      <c r="G21" s="53" t="inlineStr">
+        <is>
+          <t>https://www.cbs17.com/news/local-news/duke-energy-planning-for-natural-gas-plants-in-roxboro/</t>
+        </is>
+      </c>
+      <c r="H21" s="53" t="inlineStr">
+        <is>
+          <t>News quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="53" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B22" s="53" t="inlineStr">
+        <is>
+          <t>Stacy Hickman</t>
+        </is>
+      </c>
+      <c r="C22" s="53" t="inlineStr">
+        <is>
+          <t>Talent Acquisition Manager</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="inlineStr">
+        <is>
+          <t>Zachry Group</t>
+        </is>
+      </c>
+      <c r="E22" s="53" t="inlineStr">
+        <is>
+          <t>Site hiring</t>
+        </is>
+      </c>
+      <c r="F22" s="53" t="inlineStr"/>
+      <c r="G22" s="53" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/stacy-hickman/</t>
+        </is>
+      </c>
+      <c r="H22" s="53" t="inlineStr">
+        <is>
+          <t>LinkedIn - verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="53" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B23" s="53" t="inlineStr">
+        <is>
+          <t>Ernest Rufus</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="inlineStr">
+        <is>
+          <t>Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
+        </is>
+      </c>
+      <c r="D23" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E23" s="53" t="inlineStr">
+        <is>
+          <t>Owner project lead</t>
+        </is>
+      </c>
+      <c r="F23" s="53" t="inlineStr"/>
+      <c r="G23" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction</t>
+        </is>
+      </c>
+      <c r="H23" s="53" t="inlineStr">
+        <is>
+          <t>Official blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="53" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="inlineStr">
+        <is>
+          <t>Haley Fisackerly</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D24" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Mississippi</t>
+        </is>
+      </c>
+      <c r="E24" s="53" t="inlineStr">
+        <is>
+          <t>Executive</t>
+        </is>
+      </c>
+      <c r="F24" s="53" t="inlineStr">
+        <is>
+          <t>Media line 769-262-0745</t>
+        </is>
+      </c>
+      <c r="G24" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-mississippi-breaks-ground-on-delta-blues-advanced-power-station</t>
+        </is>
+      </c>
+      <c r="H24" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="53" t="inlineStr">
+        <is>
+          <t>Vicksburg Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B25" s="53" t="inlineStr">
+        <is>
+          <t>Ernest Rufus</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>Senior Manager, Capital Projects</t>
+        </is>
+      </c>
+      <c r="D25" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E25" s="53" t="inlineStr">
+        <is>
+          <t>Owner project lead</t>
+        </is>
+      </c>
+      <c r="F25" s="53" t="inlineStr"/>
+      <c r="G25" s="53" t="inlineStr">
+        <is>
+          <t>https://www.vicksburgpost.com/news/vicksburg-board-grants-conditional-fee-waiver-for-new-entergy-power-plant-3320f9d2</t>
+        </is>
+      </c>
+      <c r="H25" s="53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B26" s="53" t="inlineStr">
+        <is>
+          <t>John E. Niland</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>VP, New Technology &amp; Thermal Development</t>
+        </is>
+      </c>
+      <c r="D26" s="53" t="inlineStr">
+        <is>
+          <t>Invenergy</t>
+        </is>
+      </c>
+      <c r="E26" s="53" t="inlineStr">
+        <is>
+          <t>Developer lead (IURC witness)</t>
+        </is>
+      </c>
+      <c r="F26" s="53" t="inlineStr"/>
+      <c r="G26" s="53" t="inlineStr">
+        <is>
+          <t>https://www.in.gov/iurc/files/ord_46295_123025.pdf</t>
+        </is>
+      </c>
+      <c r="H26" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B27" s="53" t="inlineStr">
+        <is>
+          <t>Daniel Runyan</t>
+        </is>
+      </c>
+      <c r="C27" s="53" t="inlineStr">
+        <is>
+          <t>SVP Development</t>
+        </is>
+      </c>
+      <c r="D27" s="53" t="inlineStr">
+        <is>
+          <t>Invenergy</t>
+        </is>
+      </c>
+      <c r="E27" s="53" t="inlineStr">
+        <is>
+          <t>Developer executive</t>
+        </is>
+      </c>
+      <c r="F27" s="53" t="inlineStr"/>
+      <c r="G27" s="53" t="inlineStr">
+        <is>
+          <t>https://www.insideindianabusiness.com/articles/indiana-michigan-power-seeks-to-acquire-sullivan-county-natural-gas-plant</t>
+        </is>
+      </c>
+      <c r="H27" s="53" t="inlineStr">
+        <is>
+          <t>News quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B28" s="53" t="inlineStr">
+        <is>
+          <t>Steve Baker</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>President &amp; COO</t>
+        </is>
+      </c>
+      <c r="D28" s="53" t="inlineStr">
+        <is>
+          <t>Indiana Michigan Power (AEP)</t>
+        </is>
+      </c>
+      <c r="E28" s="53" t="inlineStr">
+        <is>
+          <t>Acquirer executive</t>
+        </is>
+      </c>
+      <c r="F28" s="53" t="inlineStr"/>
+      <c r="G28" s="53" t="inlineStr">
+        <is>
+          <t>https://www.aep.com/news/stories/view/11850/</t>
+        </is>
+      </c>
+      <c r="H28" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B29" s="53" t="inlineStr">
+        <is>
+          <t>Timothy B. Gaul</t>
+        </is>
+      </c>
+      <c r="C29" s="53" t="inlineStr">
+        <is>
+          <t>Director, Regulated Infrastructure Development</t>
+        </is>
+      </c>
+      <c r="D29" s="53" t="inlineStr">
+        <is>
+          <t>AEP Service Corp</t>
+        </is>
+      </c>
+      <c r="E29" s="53" t="inlineStr">
+        <is>
+          <t>Utility-side project lead (witness)</t>
+        </is>
+      </c>
+      <c r="F29" s="53" t="inlineStr"/>
+      <c r="G29" s="53" t="inlineStr">
+        <is>
+          <t>https://www.in.gov/iurc/files/ord_46238_091025.pdf</t>
+        </is>
+      </c>
+      <c r="H29" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B30" s="53" t="inlineStr">
+        <is>
+          <t>Timothy C. Kerns</t>
+        </is>
+      </c>
+      <c r="C30" s="53" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D30" s="53" t="inlineStr">
+        <is>
+          <t>Sterling Industrial LLC</t>
+        </is>
+      </c>
+      <c r="E30" s="53" t="inlineStr">
+        <is>
+          <t>Owner's engineer / technical witness</t>
+        </is>
+      </c>
+      <c r="F30" s="53" t="inlineStr"/>
+      <c r="G30" s="53" t="inlineStr">
+        <is>
+          <t>IURC Cause 46389 Petitioner's Exhibit 4</t>
+        </is>
+      </c>
+      <c r="H30" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="53" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B31" s="53" t="inlineStr">
+        <is>
+          <t>The Boldt Company</t>
+        </is>
+      </c>
+      <c r="C31" s="53" t="inlineStr">
+        <is>
+          <t>Constructor (role to confirm)</t>
+        </is>
+      </c>
+      <c r="D31" s="53" t="inlineStr">
+        <is>
+          <t>Boldt (Appleton, WI)</t>
+        </is>
+      </c>
+      <c r="E31" s="53" t="inlineStr">
+        <is>
+          <t>Construction Sep 2026-Feb 2029</t>
+        </is>
+      </c>
+      <c r="F31" s="53" t="inlineStr"/>
+      <c r="G31" s="53" t="inlineStr">
+        <is>
+          <t>https://www.boldt.com/discover/sycamore-riverside-energy-center/</t>
+        </is>
+      </c>
+      <c r="H31" s="53" t="inlineStr">
+        <is>
+          <t>Company website</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B32" s="53" t="inlineStr">
+        <is>
+          <t>Nicholas D. Pressler</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="inlineStr">
+        <is>
+          <t>Director, Power Development</t>
+        </is>
+      </c>
+      <c r="D32" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Services LLC</t>
+        </is>
+      </c>
+      <c r="E32" s="53" t="inlineStr">
+        <is>
+          <t>EPC/TSL selection witness</t>
+        </is>
+      </c>
+      <c r="F32" s="53" t="inlineStr"/>
+      <c r="G32" s="53" t="inlineStr">
+        <is>
+          <t>https://lpscpubvalence.lpsc.louisiana.gov/portal/PSC/ViewFile?fileId=hsljNiQroZw%3D</t>
+        </is>
+      </c>
+      <c r="H32" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B33" s="53" t="inlineStr">
+        <is>
+          <t>Phillip May</t>
+        </is>
+      </c>
+      <c r="C33" s="53" t="inlineStr">
+        <is>
+          <t>President &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D33" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Louisiana</t>
+        </is>
+      </c>
+      <c r="E33" s="53" t="inlineStr">
+        <is>
+          <t>Executive</t>
+        </is>
+      </c>
+      <c r="F33" s="53" t="inlineStr"/>
+      <c r="G33" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
+        </is>
+      </c>
+      <c r="H33" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B34" s="53" t="inlineStr">
+        <is>
+          <t>Jim Niemiec</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="inlineStr">
+        <is>
+          <t>VP &amp; Chief Supply Chain Officer</t>
+        </is>
+      </c>
+      <c r="D34" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E34" s="53" t="inlineStr">
+        <is>
+          <t>Corporate procurement</t>
+        </is>
+      </c>
+      <c r="F34" s="53" t="inlineStr"/>
+      <c r="G34" s="53" t="inlineStr">
+        <is>
+          <t>https://nudc.com/staff-and-executive-leadership/board-directors/james-nbsp-w.-nbsp-niemiec-nbsp/</t>
+        </is>
+      </c>
+      <c r="H34" s="53" t="inlineStr">
+        <is>
+          <t>Org website</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B35" s="53" t="inlineStr">
+        <is>
+          <t>Kimberly Cook-Nelson</t>
+        </is>
+      </c>
+      <c r="C35" s="53" t="inlineStr">
+        <is>
+          <t>EVP &amp; Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="D35" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E35" s="53" t="inlineStr">
+        <is>
+          <t>Generation &amp; capital projects executive</t>
+        </is>
+      </c>
+      <c r="F35" s="53" t="inlineStr"/>
+      <c r="G35" s="53" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/leadership/kimberly-cook-nelson</t>
+        </is>
+      </c>
+      <c r="H35" s="53" t="inlineStr">
+        <is>
+          <t>Official website</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B36" s="53" t="inlineStr">
+        <is>
+          <t>Brandon Scardigli</t>
+        </is>
+      </c>
+      <c r="C36" s="53" t="inlineStr">
+        <is>
+          <t>Media contact</t>
+        </is>
+      </c>
+      <c r="D36" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Louisiana</t>
+        </is>
+      </c>
+      <c r="E36" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F36" s="53" t="inlineStr">
+        <is>
+          <t>bscardi@entergy.com; 504-576-4132</t>
+        </is>
+      </c>
+      <c r="G36" s="53" t="inlineStr">
+        <is>
+          <t>https://www.opportunitylouisiana.gov/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
+        </is>
+      </c>
+      <c r="H36" s="53" t="inlineStr">
+        <is>
+          <t>Official release</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="53" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B37" s="53" t="inlineStr">
+        <is>
+          <t>Nicholas D. Pressler</t>
+        </is>
+      </c>
+      <c r="C37" s="53" t="inlineStr">
+        <is>
+          <t>Director, Power Development</t>
+        </is>
+      </c>
+      <c r="D37" s="53" t="inlineStr">
+        <is>
+          <t>Entergy Services LLC</t>
+        </is>
+      </c>
+      <c r="E37" s="53" t="inlineStr">
+        <is>
+          <t>EPC witness (Waterford 6 filing)</t>
+        </is>
+      </c>
+      <c r="F37" s="53" t="inlineStr"/>
+      <c r="G37" s="53" t="inlineStr">
+        <is>
+          <t>https://lpscpubvalence.lpsc.louisiana.gov/portal/PSC/ViewFile?fileId=hsljNiQroZw%3D</t>
+        </is>
+      </c>
+      <c r="H37" s="53" t="inlineStr">
+        <is>
+          <t>Regulatory filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B38" s="53" t="inlineStr">
+        <is>
+          <t>Michelle Berg</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="inlineStr">
+        <is>
+          <t>Entergy representative</t>
+        </is>
+      </c>
+      <c r="D38" s="53" t="inlineStr">
+        <is>
+          <t>Entergy</t>
+        </is>
+      </c>
+      <c r="E38" s="53" t="inlineStr">
+        <is>
+          <t>Parish council briefing</t>
+        </is>
+      </c>
+      <c r="F38" s="53" t="inlineStr"/>
+      <c r="G38" s="53" t="inlineStr">
+        <is>
+          <t>https://citizenportal.ai/articles/6476185/Louisiana/St-Charles-Parish/Entergy-announces-plans-for-two-new-combined-cycle-units-at-Waterford-site-cites-2B-plus-investment-and-local-jobs</t>
+        </is>
+      </c>
+      <c r="H38" s="53" t="inlineStr">
+        <is>
+          <t>Secondary source - verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="53" t="inlineStr">
+        <is>
+          <t>All Entergy program plants</t>
+        </is>
+      </c>
+      <c r="B39" s="53" t="inlineStr">
+        <is>
+          <t>TSL Power Partners (JV TIC/Kiewit + Sargent &amp; Lundy)</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>EPC procurement</t>
+        </is>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>TSL Power Partners</t>
+        </is>
+      </c>
+      <c r="E39" s="53" t="inlineStr">
+        <is>
+          <t>Buys cable for Entergy CC/CT program</t>
+        </is>
+      </c>
+      <c r="F39" s="53" t="inlineStr">
+        <is>
+          <t>8900 Renner Blvd, Lenexa, KS 66219</t>
+        </is>
+      </c>
+      <c r="G39" s="53" t="inlineStr">
+        <is>
+          <t>https://www.ticus.com/entergy-program/</t>
+        </is>
+      </c>
+      <c r="H39" s="53" t="inlineStr">
+        <is>
+          <t>Company website / customs record</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tag sales comments and descriptions with reported pipeline source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2053,7 +2053,7 @@
       </c>
       <c r="AJ7" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="AK7" s="38" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="AL7" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. EPC: Not public. OEM: GE Vernova (5x 7F.05 CTs, H35 generators). Utility: American Transmission Co (ATC); possible offtaker We Energies. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. EPC: Not public. OEM: GE Vernova (5x 7F.05 CTs, H35 generators). Utility: American Transmission Co (ATC); possible offtaker We Energies. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM7" s="40" t="n"/>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="AJ8" s="38" t="inlineStr">
         <is>
-          <t>In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="AK8" s="38" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="AL8" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. EPC: Mitsubishi Power / TIC / Sargent &amp; Lundy (EPC consortium). OEM: Mitsubishi Power (2x M501JAC GT, ST, HRSG). Utility: Entergy Texas. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. EPC: Mitsubishi Power / TIC / Sargent &amp; Lundy (EPC consortium). OEM: Mitsubishi Power (2x M501JAC GT, ST, HRSG). Utility: Entergy Texas. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM8" s="40" t="n"/>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="AJ9" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="AK9" s="38" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="AL9" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. EPC: Not public. OEM: Not found. Utility: ERCOT (West Texas). RTO: Electric Reliability Council of Texas (ERCOT).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. EPC: Not public. OEM: Not found. Utility: ERCOT (West Texas). RTO: Electric Reliability Council of Texas (ERCOT).</t>
         </is>
       </c>
       <c r="AM9" s="40" t="n"/>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="AJ10" s="38" t="inlineStr">
         <is>
-          <t>LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="AK10" s="38" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="AL10" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE).</t>
         </is>
       </c>
       <c r="AM10" s="40" t="n"/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="AJ11" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="AK11" s="38" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="AL11" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM11" s="40" t="n"/>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="AJ12" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="AK12" s="38" t="inlineStr">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="AL12" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. EPC: Zachry Group. OEM: GE Vernova (advanced-class GTs). Utility: Duke Energy Progress. RTO: Southeast (SE).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. EPC: Zachry Group. OEM: GE Vernova (advanced-class GTs). Utility: Duke Energy Progress. RTO: Southeast (SE).</t>
         </is>
       </c>
       <c r="AM12" s="40" t="n"/>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="AJ13" s="38" t="inlineStr">
         <is>
-          <t>MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="AK13" s="38" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="AL13" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. EPC: TSL Power Partners (Kiewit / TIC). OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. EPC: TSL Power Partners (Kiewit / TIC). OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM13" s="40" t="n"/>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AJ14" s="38" t="inlineStr">
         <is>
-          <t>URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="AK14" s="38" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="AL14" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM14" s="40" t="n"/>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="AJ15" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="AK15" s="38" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="AL15" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM).</t>
         </is>
       </c>
       <c r="AM15" s="40" t="n"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="AJ16" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="AK16" s="38" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AL16" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. EPC: TSL Power Partners (TIC / Sargent &amp; Lundy) with Mitsubishi Power Americas. OEM: Mitsubishi Power M501JAC (2x 1x1 CC). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. EPC: TSL Power Partners (TIC / Sargent &amp; Lundy) with Mitsubishi Power Americas. OEM: Mitsubishi Power M501JAC (2x 1x1 CC). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM16" s="40" t="n"/>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="AJ17" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="AK17" s="38" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="AL17" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
         </is>
       </c>
       <c r="AM17" s="40" t="n"/>
@@ -14843,7 +14843,7 @@
       <c r="CF7" s="39" t="n"/>
       <c r="CG7" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="CH7" s="38" t="inlineStr">
@@ -14853,7 +14853,7 @@
       </c>
       <c r="CI7" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation.</t>
         </is>
       </c>
       <c r="CJ7" s="38" t="inlineStr">
@@ -15135,7 +15135,7 @@
       <c r="CF8" s="39" t="n"/>
       <c r="CG8" s="38" t="inlineStr">
         <is>
-          <t>In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="CH8" s="38" t="inlineStr">
@@ -15145,7 +15145,7 @@
       </c>
       <c r="CI8" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026.</t>
         </is>
       </c>
       <c r="CJ8" s="38" t="inlineStr">
@@ -15423,7 +15423,7 @@
       <c r="CF9" s="39" t="n"/>
       <c r="CG9" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="CH9" s="38" t="inlineStr">
@@ -15433,7 +15433,7 @@
       </c>
       <c r="CI9" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth.</t>
         </is>
       </c>
       <c r="CJ9" s="38" t="inlineStr">
@@ -15719,7 +15719,7 @@
       <c r="CF10" s="39" t="n"/>
       <c r="CG10" s="38" t="inlineStr">
         <is>
-          <t>LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="CH10" s="38" t="inlineStr">
@@ -15729,7 +15729,7 @@
       </c>
       <c r="CI10" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027.</t>
         </is>
       </c>
       <c r="CJ10" s="38" t="inlineStr">
@@ -16011,7 +16011,7 @@
       <c r="CF11" s="39" t="n"/>
       <c r="CG11" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="CH11" s="38" t="inlineStr">
@@ -16021,7 +16021,7 @@
       </c>
       <c r="CI11" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027).</t>
         </is>
       </c>
       <c r="CJ11" s="38" t="inlineStr">
@@ -16315,7 +16315,7 @@
       <c r="CF12" s="39" t="n"/>
       <c r="CG12" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="CH12" s="38" t="inlineStr">
@@ -16325,7 +16325,7 @@
       </c>
       <c r="CI12" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind.</t>
         </is>
       </c>
       <c r="CJ12" s="38" t="inlineStr">
@@ -16621,7 +16621,7 @@
       <c r="CF13" s="39" t="n"/>
       <c r="CG13" s="38" t="inlineStr">
         <is>
-          <t>MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="CH13" s="38" t="inlineStr">
@@ -16631,7 +16631,7 @@
       </c>
       <c r="CI13" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation.</t>
         </is>
       </c>
       <c r="CJ13" s="38" t="inlineStr">
@@ -16913,7 +16913,7 @@
       <c r="CF14" s="39" t="n"/>
       <c r="CG14" s="38" t="inlineStr">
         <is>
-          <t>URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="CH14" s="38" t="inlineStr">
@@ -16923,7 +16923,7 @@
       </c>
       <c r="CI14" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus.</t>
         </is>
       </c>
       <c r="CJ14" s="38" t="inlineStr">
@@ -17207,7 +17207,7 @@
       <c r="CF15" s="39" t="n"/>
       <c r="CG15" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="CH15" s="38" t="inlineStr">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="CI15" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station.</t>
         </is>
       </c>
       <c r="CJ15" s="38" t="inlineStr">
@@ -17501,7 +17501,7 @@
       <c r="CF16" s="39" t="n"/>
       <c r="CG16" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="CH16" s="38" t="inlineStr">
@@ -17511,7 +17511,7 @@
       </c>
       <c r="CI16" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years.</t>
         </is>
       </c>
       <c r="CJ16" s="38" t="inlineStr">
@@ -17805,7 +17805,7 @@
       <c r="CF17" s="39" t="n"/>
       <c r="CG17" s="38" t="inlineStr">
         <is>
-          <t>CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="CH17" s="38" t="inlineStr">
@@ -17815,7 +17815,7 @@
       </c>
       <c r="CI17" s="38" t="inlineStr">
         <is>
-          <t>Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load.</t>
         </is>
       </c>
       <c r="CJ17" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Add source reference links to project descriptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2063,7 +2063,7 @@
       </c>
       <c r="AL7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. EPC: Not public. OEM: GE Vernova (5x 7F.05 CTs, H35 generators). Utility: American Transmission Co (ATC); possible offtaker We Energies. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. EPC: Not public. OEM: GE Vernova (5x 7F.05 CTs, H35 generators). Utility: American Transmission Co (ATC); possible offtaker We Energies. RTO: Midcontinent Independent System Operator (MISO). Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="AM7" s="40" t="n"/>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="AL8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. EPC: Mitsubishi Power / TIC / Sargent &amp; Lundy (EPC consortium). OEM: Mitsubishi Power (2x M501JAC GT, ST, HRSG). Utility: Entergy Texas. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. EPC: Mitsubishi Power / TIC / Sargent &amp; Lundy (EPC consortium). OEM: Mitsubishi Power (2x M501JAC GT, ST, HRSG). Utility: Entergy Texas. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="AM8" s="40" t="n"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="AL9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. EPC: Not public. OEM: Not found. Utility: ERCOT (West Texas). RTO: Electric Reliability Council of Texas (ERCOT).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. EPC: Not public. OEM: Not found. Utility: ERCOT (West Texas). RTO: Electric Reliability Council of Texas (ERCOT). Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="AM9" s="40" t="n"/>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="AL10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE). Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="AM10" s="40" t="n"/>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="AL11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="AM11" s="40" t="n"/>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="AL12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. EPC: Zachry Group. OEM: GE Vernova (advanced-class GTs). Utility: Duke Energy Progress. RTO: Southeast (SE).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. EPC: Zachry Group. OEM: GE Vernova (advanced-class GTs). Utility: Duke Energy Progress. RTO: Southeast (SE). Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="AM12" s="40" t="n"/>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="AL13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. EPC: TSL Power Partners (Kiewit / TIC). OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. EPC: TSL Power Partners (Kiewit / TIC). OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="AM13" s="40" t="n"/>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="AL14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="AM14" s="40" t="n"/>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="AL15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM). Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="AM15" s="40" t="n"/>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AL16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. EPC: TSL Power Partners (TIC / Sargent &amp; Lundy) with Mitsubishi Power Americas. OEM: Mitsubishi Power M501JAC (2x 1x1 CC). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. EPC: TSL Power Partners (TIC / Sargent &amp; Lundy) with Mitsubishi Power Americas. OEM: Mitsubishi Power M501JAC (2x 1x1 CC). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="AM16" s="40" t="n"/>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="AL17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="AM17" s="40" t="n"/>
@@ -13502,10 +13502,23 @@
       <formula1>YesNo</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL17" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
@@ -14853,7 +14866,7 @@
       </c>
       <c r="CI7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="CJ7" s="38" t="inlineStr">
@@ -15145,7 +15158,7 @@
       </c>
       <c r="CI8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="CJ8" s="38" t="inlineStr">
@@ -15433,7 +15446,7 @@
       </c>
       <c r="CI9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="CJ9" s="38" t="inlineStr">
@@ -15729,7 +15742,7 @@
       </c>
       <c r="CI10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="CJ10" s="38" t="inlineStr">
@@ -16021,7 +16034,7 @@
       </c>
       <c r="CI11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027).</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="CJ11" s="38" t="inlineStr">
@@ -16325,7 +16338,7 @@
       </c>
       <c r="CI12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="CJ12" s="38" t="inlineStr">
@@ -16631,7 +16644,7 @@
       </c>
       <c r="CI13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="CJ13" s="38" t="inlineStr">
@@ -16923,7 +16936,7 @@
       </c>
       <c r="CI14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="CJ14" s="38" t="inlineStr">
@@ -17217,7 +17230,7 @@
       </c>
       <c r="CI15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="CJ15" s="38" t="inlineStr">
@@ -17511,7 +17524,7 @@
       </c>
       <c r="CI16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="CJ16" s="38" t="inlineStr">
@@ -17815,7 +17828,7 @@
       </c>
       <c r="CI17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load.</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="CJ17" s="38" t="inlineStr">
@@ -34948,10 +34961,23 @@
       <formula1>YesNo</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI17" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Expand project descriptions with technology, site, equipment and W&C needs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2063,7 +2063,7 @@
       </c>
       <c r="AL7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. EPC: Not public. OEM: GE Vernova (5x 7F.05 CTs, H35 generators). Utility: American Transmission Co (ATC); possible offtaker We Energies. RTO: Midcontinent Independent System Operator (MISO). Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. RTO: Midcontinent Independent System Operator (MISO). Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="AM7" s="40" t="n"/>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="AL8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. EPC: Mitsubishi Power / TIC / Sargent &amp; Lundy (EPC consortium). OEM: Mitsubishi Power (2x M501JAC GT, ST, HRSG). Utility: Entergy Texas. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="AM8" s="40" t="n"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="AL9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. EPC: Not public. OEM: Not found. Utility: ERCOT (West Texas). RTO: Electric Reliability Council of Texas (ERCOT). Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. RTO: Electric Reliability Council of Texas (ERCOT). Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="AM9" s="40" t="n"/>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="AL10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. EPC: Mitsubishi Power Americas + Black &amp; Veatch Construction (EPC consortium, contract 1/12/2024). OEM: Mitsubishi Power M501JAC CTs; Mitsubishi Electric VP-X generators. Utility: Georgia Power. RTO: Southeast (SE). Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. RTO: Southeast (SE). Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="AM10" s="40" t="n"/>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="AL11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Mitsubishi Power (implied by TSL/MPWA program). Utility: Entergy Arkansas. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="AM11" s="40" t="n"/>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="AL12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. EPC: Zachry Group. OEM: GE Vernova (advanced-class GTs). Utility: Duke Energy Progress. RTO: Southeast (SE). Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. RTO: Southeast (SE). Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="AM12" s="40" t="n"/>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="AL13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. EPC: TSL Power Partners (Kiewit / TIC). OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="AM13" s="40" t="n"/>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="AL14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. EPC: TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). OEM: Unverified (Yes Energy: Mitsubishi). Utility: Entergy Mississippi. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="AM14" s="40" t="n"/>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="AL15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. EPC: The Boldt Company (constructor per Boldt project page - role to confirm). OEM: GE Vernova (4x 7F.05 CTs). Utility: Indiana Michigan Power (AEP). RTO: PJM Interconnection (PJM). Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. RTO: PJM Interconnection (PJM). Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="AM15" s="40" t="n"/>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AL16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. EPC: TSL Power Partners (TIC / Sargent &amp; Lundy) with Mitsubishi Power Americas. OEM: Mitsubishi Power M501JAC (2x 1x1 CC). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="AM16" s="40" t="n"/>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="AL17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. EPC: TSL Power Partners (TIC + Sargent &amp; Lundy) - implied by LPSC Waterford 6 filing. OEM: Mitsubishi Power M501JAC (per GEM). Utility: Entergy Louisiana. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="AM17" s="40" t="n"/>
@@ -14866,7 +14866,7 @@
       </c>
       <c r="CI7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. ~1.2 GW simple-cycle peaker (5x GE 7F.05) next to the proposed 750 MW Union Depot CC (~1.95 GW combined). Three 345 kV overhead gen-ties to ATC Forest Junction substation. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="CJ7" s="38" t="inlineStr">
@@ -15158,7 +15158,7 @@
       </c>
       <c r="CI8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. 1,215 MW hydrogen-capable 2x1 combined cycle at the Sabine site, built by Mitsubishi/TIC/S&amp;L consortium. Online Oct 2026. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="CJ8" s="38" t="inlineStr">
@@ -15446,7 +15446,7 @@
       </c>
       <c r="CI9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. Two dual-fuel simple-cycle CTs (~860 MW total; Unit I ~440 MW) at the existing Permian Basin Power Plant, raising site to 1,185 MW. Serves Permian oil &amp; gas load growth. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="CJ9" s="38" t="inlineStr">
@@ -15742,7 +15742,7 @@
       </c>
       <c r="CI10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. Three simple-cycle dual-fuel M501JAC units (~1.3 GW) at existing Plant Yates; Unit 8 Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="CJ10" s="38" t="inlineStr">
@@ -16034,7 +16034,7 @@
       </c>
       <c r="CI11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. 446 MW hydrogen-capable simple-cycle CT on ~20 acres of the Lake Catherine site, replacing Lake Catherine Unit 4 (retiring end-2027). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="CJ11" s="38" t="inlineStr">
@@ -16338,7 +16338,7 @@
       </c>
       <c r="CI12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. 1,360 MW 2x1 hydrogen-capable GE Vernova combined cycle at Duke's Roxboro coal site, full EPC by Zachry; identical CC2 ~1 year behind. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="CJ12" s="38" t="inlineStr">
@@ -16644,7 +16644,7 @@
       </c>
       <c r="CI13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable combined cycle replacing the 1950s Andrus plant in Greenville; ~1.5 mi new transmission line to existing substation. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="CJ13" s="38" t="inlineStr">
@@ -16936,7 +16936,7 @@
       </c>
       <c r="CI14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. 754 MW hydrogen-capable, carbon-capture-enabled combined cycle on the demolished Baxter Wilson site; tied contextually to the AWS $3B Vicksburg data center campus. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="CJ14" s="38" t="inlineStr">
@@ -17230,7 +17230,7 @@
       </c>
       <c r="CI15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. ~918-935 MW simple-cycle peaker (4x GE 7F.05) developed by Invenergy, acquired by I&amp;M at COD (Mar 2029); interconnects at AEP Sullivan 345 kV station. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="CJ15" s="38" t="inlineStr">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="CI16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. Two 1x1 hydrogen-capable combined-cycle units (~1.5 GW) serving Meta's Hyperion AI data center campus; Meta pays full revenue requirement for 15 years. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="CJ16" s="38" t="inlineStr">
@@ -17828,7 +17828,7 @@
       </c>
       <c r="CI17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. 1x1 Mitsubishi M501JAC combined cycle on Entergy's existing Waterford site (Waterford 1-3), 500 kV interconnection; supports Meta Hyperion load. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="CJ17" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Remove description hyperlinks; make source links clickable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -49,7 +49,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -84,6 +84,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -132,10 +139,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -293,9 +301,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="7">
     <dxf>
@@ -13502,23 +13515,10 @@
       <formula1>YesNo</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL17" r:id="rId11"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -34961,23 +34961,10 @@
       <formula1>YesNo</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="CI17" r:id="rId11"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -44348,11 +44335,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="160" customWidth="1" min="2" max="2"/>
+    <col width="140" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44363,143 +44350,507 @@
       </c>
       <c r="B1" s="53" t="inlineStr">
         <is>
-          <t>Key sources (web research 10/29/2026)</t>
+          <t>Source link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Forest Junction Energy Center</t>
         </is>
       </c>
-      <c r="B2" s="54" t="inlineStr">
-        <is>
-          <t>https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ ; https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot ; https://forestjunctionenergycenter.invenergy.com/ ; https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+      <c r="B2" s="55" t="inlineStr">
+        <is>
+          <t>https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="54" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B3" s="55" t="inlineStr">
+        <is>
+          <t>https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="inlineStr">
+        <is>
+          <t>https://forestjunctionenergycenter.invenergy.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Orange County Advanced Power Station (OCAPS)</t>
         </is>
       </c>
-      <c r="B3" s="54" t="inlineStr">
-        <is>
-          <t>https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ ; https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ ; https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="54" t="inlineStr">
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="inlineStr">
+        <is>
+          <t>https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
         </is>
       </c>
-      <c r="B4" s="54" t="inlineStr">
-        <is>
-          <t>https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas ; https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin ; https://www.gem.wiki/Permian_Power_power_station ; https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="54" t="inlineStr">
+      <c r="B9" s="55" t="inlineStr">
+        <is>
+          <t>https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B11" s="55" t="inlineStr">
+        <is>
+          <t>https://www.gem.wiki/Permian_Power_power_station</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="inlineStr">
+        <is>
+          <t>https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
         </is>
       </c>
-      <c r="B5" s="54" t="inlineStr">
-        <is>
-          <t>https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html ; https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf ; https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="54" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B14" s="55" t="inlineStr">
+        <is>
+          <t>https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="inlineStr">
+        <is>
+          <t>https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Ironwood Power Station</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
-        <is>
-          <t>https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station ; https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ ; https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="54" t="inlineStr">
+      <c r="B16" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="inlineStr">
+        <is>
+          <t>https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B18" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Person County Combined Cycle 1 (CC1)</t>
         </is>
       </c>
-      <c r="B7" s="54" t="inlineStr">
-        <is>
-          <t>https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html ; https://www.duke-energy.com/info/person ; https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="54" t="inlineStr">
+      <c r="B19" s="55" t="inlineStr">
+        <is>
+          <t>https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B20" s="55" t="inlineStr">
+        <is>
+          <t>https://www.duke-energy.com/info/person</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t>https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Delta Blues Advanced Power Station</t>
         </is>
       </c>
-      <c r="B8" s="54" t="inlineStr">
-        <is>
-          <t>https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ ; https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction ; https://www.gem.wiki/Delta_Blues_Advanced_Power_Station ; https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t>https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B23" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B24" s="55" t="inlineStr">
+        <is>
+          <t>https://www.gem.wiki/Delta_Blues_Advanced_Power_Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Vicksburg Advanced Power Station</t>
         </is>
       </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>https://www.entergymississippi.com/generation/vicksburg ; https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ ; https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="54" t="inlineStr">
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergymississippi.com/generation/vicksburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Vicksburg Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t>https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Vicksburg Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B28" s="55" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Sycamore Riverside Energy Center</t>
         </is>
       </c>
-      <c r="B10" s="54" t="inlineStr">
-        <is>
-          <t>https://www.aep.com/news/stories/view/11850/ ; https://sycamoreriverside.invenergy.com/about-project ; https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf ; https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="54" t="inlineStr">
+      <c r="B29" s="55" t="inlineStr">
+        <is>
+          <t>https://www.aep.com/news/stories/view/11850/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B30" s="55" t="inlineStr">
+        <is>
+          <t>https://sycamoreriverside.invenergy.com/about-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B31" s="55" t="inlineStr">
+        <is>
+          <t>https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B32" s="55" t="inlineStr">
+        <is>
+          <t>https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
-        <is>
-          <t>https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation ; https://www.ticus.com/entergy-program/ ; https://www.gem.wiki/Franklin_Farms_power_station ; https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
+      <c r="B33" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B34" s="55" t="inlineStr">
+        <is>
+          <t>https://www.ticus.com/entergy-program/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B35" s="55" t="inlineStr">
+        <is>
+          <t>https://www.gem.wiki/Franklin_Farms_power_station</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B36" s="55" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Waterford 5 Power Station</t>
         </is>
       </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>https://www.entergylouisiana.com/waterford5-6 ; https://www.interconnection.fyi/project/miso-e0029 ; https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+      <c r="B37" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergylouisiana.com/waterford5-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B38" s="55" t="inlineStr">
+        <is>
+          <t>https://www.interconnection.fyi/project/miso-e0029</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B39" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -44592,7 +44943,7 @@
         </is>
       </c>
       <c r="F2" s="54" t="inlineStr"/>
-      <c r="G2" s="54" t="inlineStr">
+      <c r="G2" s="56" t="inlineStr">
         <is>
           <t>https://www.nbc26.com/lakeshore/two-natural-gas-power-plants-proposed-in-brillion</t>
         </is>
@@ -44630,7 +44981,7 @@
         </is>
       </c>
       <c r="F3" s="54" t="inlineStr"/>
-      <c r="G3" s="54" t="inlineStr">
+      <c r="G3" s="56" t="inlineStr">
         <is>
           <t>https://www.wpr.org/news/energy-developer-planning-2-gigawatt-natural-gas-plants-northeast-wisconsin</t>
         </is>
@@ -44668,7 +45019,7 @@
         </is>
       </c>
       <c r="F4" s="54" t="inlineStr"/>
-      <c r="G4" s="54" t="inlineStr">
+      <c r="G4" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/news/construction-nears-completion-on-entergy-texas-orange-county-advanced-power-station</t>
         </is>
@@ -44706,7 +45057,7 @@
         </is>
       </c>
       <c r="F5" s="54" t="inlineStr"/>
-      <c r="G5" s="54" t="inlineStr">
+      <c r="G5" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/news/entergy-texas-orange-county-advanced-power-station-begins-delivering-reliable-power-to-southeast-texas</t>
         </is>
@@ -44744,7 +45095,7 @@
         </is>
       </c>
       <c r="F6" s="54" t="inlineStr"/>
-      <c r="G6" s="54" t="inlineStr">
+      <c r="G6" s="56" t="inlineStr">
         <is>
           <t>https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
@@ -44786,7 +45137,7 @@
           <t>Media line 281-297-2353</t>
         </is>
       </c>
-      <c r="G7" s="54" t="inlineStr">
+      <c r="G7" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/news/media-kit</t>
         </is>
@@ -44824,7 +45175,7 @@
         </is>
       </c>
       <c r="F8" s="54" t="inlineStr"/>
-      <c r="G8" s="54" t="inlineStr">
+      <c r="G8" s="56" t="inlineStr">
         <is>
           <t>https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas</t>
         </is>
@@ -44862,7 +45213,7 @@
         </is>
       </c>
       <c r="F9" s="54" t="inlineStr"/>
-      <c r="G9" s="54" t="inlineStr">
+      <c r="G9" s="56" t="inlineStr">
         <is>
           <t>https://www.georgiapower.com/news-hub/press-releases/first-new-natural-gas-turbine-delivered-to-georgia-power-plant-yates.html</t>
         </is>
@@ -44900,7 +45251,7 @@
         </is>
       </c>
       <c r="F10" s="54" t="inlineStr"/>
-      <c r="G10" s="54" t="inlineStr">
+      <c r="G10" s="56" t="inlineStr">
         <is>
           <t>https://power.mhi.com/regions/amer/news/250819</t>
         </is>
@@ -44938,7 +45289,7 @@
         </is>
       </c>
       <c r="F11" s="54" t="inlineStr"/>
-      <c r="G11" s="54" t="inlineStr">
+      <c r="G11" s="56" t="inlineStr">
         <is>
           <t>https://www.bv.com/en-US/projects/gas-fired-power-plant-project-defies-challenges-to-deliver-safe-reliable-power</t>
         </is>
@@ -44976,7 +45327,7 @@
         </is>
       </c>
       <c r="F12" s="54" t="inlineStr"/>
-      <c r="G12" s="54" t="inlineStr">
+      <c r="G12" s="56" t="inlineStr">
         <is>
           <t>https://apps.apsc.arkansas.gov/pdf/24/24-072-U_67_1.pdf</t>
         </is>
@@ -45014,7 +45365,7 @@
         </is>
       </c>
       <c r="F13" s="54" t="inlineStr"/>
-      <c r="G13" s="54" t="inlineStr">
+      <c r="G13" s="56" t="inlineStr">
         <is>
           <t>https://www.arkansasonline.com/news/2026/aug/21/entergy-breaks-ground-on-ironwood-power-station/</t>
         </is>
@@ -45052,7 +45403,7 @@
         </is>
       </c>
       <c r="F14" s="54" t="inlineStr"/>
-      <c r="G14" s="54" t="inlineStr">
+      <c r="G14" s="56" t="inlineStr">
         <is>
           <t>https://adeq.state.ar.us/downloads/WebDatabases/PermitsOnline/NPDES/PermitInformation/AR0001147_Certificate%20of%20Service%20Letter_20260430.pdf</t>
         </is>
@@ -45094,7 +45445,7 @@
           <t>wmcmast@entergy.com (ADEQ permit)</t>
         </is>
       </c>
-      <c r="G15" s="54" t="inlineStr">
+      <c r="G15" s="56" t="inlineStr">
         <is>
           <t>https://adeq.state.ar.us/downloads/WebDatabases/PermitsOnline/Air/1717-AOP-R9.pdf</t>
         </is>
@@ -45132,7 +45483,7 @@
         </is>
       </c>
       <c r="F16" s="54" t="inlineStr"/>
-      <c r="G16" s="54" t="inlineStr">
+      <c r="G16" s="56" t="inlineStr">
         <is>
           <t>https://arkansasstatechamber.com/team-member/kendall-thornton/</t>
         </is>
@@ -45170,7 +45521,7 @@
         </is>
       </c>
       <c r="F17" s="54" t="inlineStr"/>
-      <c r="G17" s="54" t="inlineStr">
+      <c r="G17" s="56" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/reesjason/</t>
         </is>
@@ -45212,7 +45563,7 @@
           <t>esupplier@entergy.com; 844-387-9675</t>
         </is>
       </c>
-      <c r="G18" s="54" t="inlineStr">
+      <c r="G18" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/suppliers/how</t>
         </is>
@@ -45250,7 +45601,7 @@
         </is>
       </c>
       <c r="F19" s="54" t="inlineStr"/>
-      <c r="G19" s="54" t="inlineStr">
+      <c r="G19" s="56" t="inlineStr">
         <is>
           <t>https://starw1.ncuc.gov/NCUC/ViewFile.aspx?Id=5552fef5-9b1f-4e88-b9ca-0e649dafdbb5</t>
         </is>
@@ -45288,7 +45639,7 @@
         </is>
       </c>
       <c r="F20" s="54" t="inlineStr"/>
-      <c r="G20" s="54" t="inlineStr">
+      <c r="G20" s="56" t="inlineStr">
         <is>
           <t>https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html</t>
         </is>
@@ -45326,7 +45677,7 @@
         </is>
       </c>
       <c r="F21" s="54" t="inlineStr"/>
-      <c r="G21" s="54" t="inlineStr">
+      <c r="G21" s="56" t="inlineStr">
         <is>
           <t>https://www.cbs17.com/news/local-news/duke-energy-planning-for-natural-gas-plants-in-roxboro/</t>
         </is>
@@ -45364,7 +45715,7 @@
         </is>
       </c>
       <c r="F22" s="54" t="inlineStr"/>
-      <c r="G22" s="54" t="inlineStr">
+      <c r="G22" s="56" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/stacy-hickman/</t>
         </is>
@@ -45402,7 +45753,7 @@
         </is>
       </c>
       <c r="F23" s="54" t="inlineStr"/>
-      <c r="G23" s="54" t="inlineStr">
+      <c r="G23" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction</t>
         </is>
@@ -45444,7 +45795,7 @@
           <t>Media line 769-262-0745</t>
         </is>
       </c>
-      <c r="G24" s="54" t="inlineStr">
+      <c r="G24" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/news/entergy-mississippi-breaks-ground-on-delta-blues-advanced-power-station</t>
         </is>
@@ -45482,7 +45833,7 @@
         </is>
       </c>
       <c r="F25" s="54" t="inlineStr"/>
-      <c r="G25" s="54" t="inlineStr">
+      <c r="G25" s="56" t="inlineStr">
         <is>
           <t>https://www.vicksburgpost.com/news/vicksburg-board-grants-conditional-fee-waiver-for-new-entergy-power-plant-3320f9d2</t>
         </is>
@@ -45520,7 +45871,7 @@
         </is>
       </c>
       <c r="F26" s="54" t="inlineStr"/>
-      <c r="G26" s="54" t="inlineStr">
+      <c r="G26" s="56" t="inlineStr">
         <is>
           <t>https://www.in.gov/iurc/files/ord_46295_123025.pdf</t>
         </is>
@@ -45558,7 +45909,7 @@
         </is>
       </c>
       <c r="F27" s="54" t="inlineStr"/>
-      <c r="G27" s="54" t="inlineStr">
+      <c r="G27" s="56" t="inlineStr">
         <is>
           <t>https://www.insideindianabusiness.com/articles/indiana-michigan-power-seeks-to-acquire-sullivan-county-natural-gas-plant</t>
         </is>
@@ -45596,7 +45947,7 @@
         </is>
       </c>
       <c r="F28" s="54" t="inlineStr"/>
-      <c r="G28" s="54" t="inlineStr">
+      <c r="G28" s="56" t="inlineStr">
         <is>
           <t>https://www.aep.com/news/stories/view/11850/</t>
         </is>
@@ -45634,7 +45985,7 @@
         </is>
       </c>
       <c r="F29" s="54" t="inlineStr"/>
-      <c r="G29" s="54" t="inlineStr">
+      <c r="G29" s="56" t="inlineStr">
         <is>
           <t>https://www.in.gov/iurc/files/ord_46238_091025.pdf</t>
         </is>
@@ -45710,7 +46061,7 @@
         </is>
       </c>
       <c r="F31" s="54" t="inlineStr"/>
-      <c r="G31" s="54" t="inlineStr">
+      <c r="G31" s="56" t="inlineStr">
         <is>
           <t>https://www.boldt.com/discover/sycamore-riverside-energy-center/</t>
         </is>
@@ -45748,7 +46099,7 @@
         </is>
       </c>
       <c r="F32" s="54" t="inlineStr"/>
-      <c r="G32" s="54" t="inlineStr">
+      <c r="G32" s="56" t="inlineStr">
         <is>
           <t>https://lpscpubvalence.lpsc.louisiana.gov/portal/PSC/ViewFile?fileId=hsljNiQroZw%3D</t>
         </is>
@@ -45786,7 +46137,7 @@
         </is>
       </c>
       <c r="F33" s="54" t="inlineStr"/>
-      <c r="G33" s="54" t="inlineStr">
+      <c r="G33" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
         </is>
@@ -45824,7 +46175,7 @@
         </is>
       </c>
       <c r="F34" s="54" t="inlineStr"/>
-      <c r="G34" s="54" t="inlineStr">
+      <c r="G34" s="56" t="inlineStr">
         <is>
           <t>https://nudc.com/staff-and-executive-leadership/board-directors/james-nbsp-w.-nbsp-niemiec-nbsp/</t>
         </is>
@@ -45862,7 +46213,7 @@
         </is>
       </c>
       <c r="F35" s="54" t="inlineStr"/>
-      <c r="G35" s="54" t="inlineStr">
+      <c r="G35" s="56" t="inlineStr">
         <is>
           <t>https://www.entergy.com/leadership/kimberly-cook-nelson</t>
         </is>
@@ -45904,7 +46255,7 @@
           <t>bscardi@entergy.com; 504-576-4132</t>
         </is>
       </c>
-      <c r="G36" s="54" t="inlineStr">
+      <c r="G36" s="56" t="inlineStr">
         <is>
           <t>https://www.opportunitylouisiana.gov/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
         </is>
@@ -45942,7 +46293,7 @@
         </is>
       </c>
       <c r="F37" s="54" t="inlineStr"/>
-      <c r="G37" s="54" t="inlineStr">
+      <c r="G37" s="56" t="inlineStr">
         <is>
           <t>https://lpscpubvalence.lpsc.louisiana.gov/portal/PSC/ViewFile?fileId=hsljNiQroZw%3D</t>
         </is>
@@ -45980,7 +46331,7 @@
         </is>
       </c>
       <c r="F38" s="54" t="inlineStr"/>
-      <c r="G38" s="54" t="inlineStr">
+      <c r="G38" s="56" t="inlineStr">
         <is>
           <t>https://citizenportal.ai/articles/6476185/Louisiana/St-Charles-Parish/Entergy-announces-plans-for-two-new-combined-cycle-units-at-Waterford-site-cites-2B-plus-investment-and-local-jobs</t>
         </is>
@@ -46022,7 +46373,7 @@
           <t>8900 Renner Blvd, Lenexa, KS 66219</t>
         </is>
       </c>
-      <c r="G39" s="54" t="inlineStr">
+      <c r="G39" s="56" t="inlineStr">
         <is>
           <t>https://www.ticus.com/entergy-program/</t>
         </is>
@@ -46034,6 +46385,45 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId37"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use *RPBD* prefix and drop filter text from descriptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2066,7 +2066,7 @@
       </c>
       <c r="AJ7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*RPBD* CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="AK7" s="38" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="AL7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. RTO: Midcontinent Independent System Operator (MISO). Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+          <t>*RPBD* OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. INVESTMENT: Total project investment Not disclosed; est. W&amp;C value $9,624,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="AM7" s="40" t="n"/>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="AJ8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="AK8" s="38" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="AL8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+          <t>*RPBD* OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. INVESTMENT: Total project investment ~$1.2B (power-eng.com); Yes Energy $555M not confirmed; est. W&amp;C value $9,720,000 ($8/kW). W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="AM8" s="40" t="n"/>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="AJ9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*RPBD* CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="AK9" s="38" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="AL9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. RTO: Electric Reliability Council of Texas (ERCOT). Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
+          <t>*RPBD* OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. INVESTMENT: Total project investment Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026); est. W&amp;C value $3,520,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="AM9" s="40" t="n"/>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="AJ10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="AK10" s="38" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="AL10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. RTO: Southeast (SE). Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
+          <t>*RPBD* OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. INVESTMENT: Total project investment Not public; PSC staff ~$1B for 3 units; est. W&amp;C value $3,862,400 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="AM10" s="40" t="n"/>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="AJ11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*RPBD* CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="AK11" s="38" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="AL11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
+          <t>*RPBD* OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). INVESTMENT: Total project investment Not disclosed (GAJA rider); est. W&amp;C value $3,568,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="AM11" s="40" t="n"/>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="AJ12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*RPBD* CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="AK12" s="38" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="AL12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. RTO: Southeast (SE). Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
+          <t>*RPBD* OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. INVESTMENT: Total project investment ~$2.13B (CC1, DEP Class 3 estimate); est. W&amp;C value $10,880,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="AM12" s="40" t="n"/>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="AJ13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
+          <t>*RPBD* MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="AK13" s="38" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="AL13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="AM13" s="40" t="n"/>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="AJ14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
+          <t>*RPBD* URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="AK14" s="38" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="AL14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $700M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="AM14" s="40" t="n"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="AJ15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*RPBD* CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="AK15" s="38" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="AL15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. RTO: PJM Interconnection (PJM). Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
+          <t>*RPBD* OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). INVESTMENT: Total project investment ~$500M capital investment (Invenergy); est. W&amp;C value $7,344,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="AM15" s="40" t="n"/>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="AJ16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*RPBD* CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="AK16" s="38" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AL16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*RPBD* OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,000,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="AM16" s="40" t="n"/>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="AJ17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*RPBD* CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="AK17" s="38" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="AL17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. RTO: Midcontinent Independent System Operator (MISO). Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+          <t>*RPBD* OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. INVESTMENT: Total project investment ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed; est. W&amp;C value $6,560,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="AM17" s="40" t="n"/>
@@ -14856,7 +14856,7 @@
       <c r="CF7" s="39" t="n"/>
       <c r="CG7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*RPBD* CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="CH7" s="38" t="inlineStr">
@@ -14866,12 +14866,12 @@
       </c>
       <c r="CI7" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019673557). Total project investment: Not disclosed. W&amp;C value (est. $8/kW): $9,624,000. OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
+          <t>*RPBD* OVERVIEW: Proposed ~1,203 MW natural-gas simple-cycle PEAKING plant by Invenergy, planned alongside the 750 MW Union Depot Energy Center combined cycle on an adjacent site (~1.95 GW total campus). Alternate site identified in Town of Woodville. TECHNOLOGY &amp; EQUIPMENT: 5x GE 7F.05 combustion turbines with GE H35 generators, each with generator step-up transformer; designed for continuous duty but expected to run mainly at peak. SITE: GREENFIELD - privately owned agricultural land east of WI-57, north of US-10, Town of Brillion, Calumet County (acreage not yet published; see PSC engineering plan). INTERCONNECTION: three 345 kV overhead gen-tie lines to ATC's Forest Junction 345 kV substation (ATC also expanding 345 kV lines south to new Sheboygan River substation). OWNERSHIP/STATUS: Developer Invenergy; We Energies listed it in rate-case planning (possible acquirer, needs PSC approval). Engineering plan filed Aug 2026; CPCN application expected fall 2026 (PSC docket 5-CE-162); construction start targeted Q4 2027; COD ~Dec 2031. EPC not yet selected. INVESTMENT: Total project investment Not disclosed; est. W&amp;C value $9,624,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Plus overhead conductor for 3x 345 kV gen-ties; large opportunity if bundled with Union Depot CC. Ref: https://dailyreporter.com/2026/08/31/invenergy-proposes-two-natural-gas-plants-calumet-county/ | https://fox11online.com/news/local/calumet-county-power-plant-proposed-energy-centers-town-of-brillion-power-megawatts-gigawatts-we-energies-invenergy-town-of-woodville-forest-junction-union-depot | https://forestjunctionenergycenter.invenergy.com/ | https://www.nbc26.com/lakeshore/neighbors-push-back-against-proposed-natural-gas-facility-in-town-of-brillion</t>
         </is>
       </c>
       <c r="CJ7" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $9,624,000 ($8/kW x 1,203 MW). Total project investment: Not disclosed.</t>
+          <t>*RPBD* Total project investment: Not disclosed. Est. W&amp;C value: $9,624,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -15148,7 +15148,7 @@
       <c r="CF8" s="39" t="n"/>
       <c r="CG8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="CH8" s="38" t="inlineStr">
@@ -15158,12 +15158,12 @@
       </c>
       <c r="CI8" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017200239). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. W&amp;C value (est. $8/kW): $9,720,000. OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
+          <t>*RPBD* OVERVIEW: 1,215 MW natural-gas COMBINED-CYCLE plant, Entergy Texas' newest unit; entered commercial service Oct 14, 2026; serves ~230,000 homes in industrial Southeast Texas. TECHNOLOGY &amp; EQUIPMENT: Mitsubishi Power powertrain - 2x M501JAC gas turbines, HRSGs and steam turbine (2x1 configuration); dual-fuel, hydrogen-capable (30% H2 at start, designed for up to 100%). SITE: BROWNFIELD - ~26.2-acre footprint inside/adjacent to Entergy Texas' existing Sabine Power Plant in Bridge City, Orange County (existing gas plant with transmission and water infrastructure). OWNERSHIP/EPC: Entergy Texas; EPC consortium Mitsubishi Power (powertrain), Sargent &amp; Lundy (engineer of record), TIC - The Industrial Company (constructor). STATUS: Construction Apr 2023-2026, first fire Apr 2026, in service Oct 2026. INVESTMENT: Total project investment ~$1.2B (power-eng.com); Yes Energy $555M not confirmed; est. W&amp;C value $9,720,000 ($8/kW). W&amp;C NEEDS: New-build cable scope complete. Remaining: MRO/spares (MV, 600V, tray &amp; instrumentation cable), outage and warranty/punch-list work; reference project for the same TIC/S&amp;L/Mitsubishi team now building Entergy's LA/MS/AR plants. Ref: https://www.click2houston.com/news/local/2026/10/14/entergy-texas-orange-county-advanced-power-station-now-delivering-power-to-southeast-texas/ | https://www.power-eng.com/gas/turbines/entergy-texas-1-2-gw-ccgt-plant-is-now-online/ | https://www.sargentlundy.com/projects/orange-county-advanced-power-station/</t>
         </is>
       </c>
       <c r="CJ8" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $9,720,000 ($8/kW x 1,215 MW). Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed.</t>
+          <t>*RPBD* Total project investment: ~$1.2B (power-eng.com); Yes Energy $555M not confirmed. Est. W&amp;C value: $9,720,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -15436,7 +15436,7 @@
       <c r="CF9" s="39" t="n"/>
       <c r="CG9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*RPBD* CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="CH9" s="38" t="inlineStr">
@@ -15446,12 +15446,12 @@
       </c>
       <c r="CI9" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018470514). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). W&amp;C value (est. $8/kW): $3,520,000. OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
+          <t>*RPBD* OVERVIEW: Vistra/Luminant expansion of the existing Permian Basin Power Plant in Monahans - two new large natural-gas SIMPLE-CYCLE units totaling 860 MW (ERCOT queue: Vast Sands Power I 28INR0105 and II 28INR0109, ~440 MW each), taking the site from 325 MW to 1,185 MW. Driven by Permian oil &amp; gas load growth. TECHNOLOGY &amp; EQUIPMENT: 2x dual-fuel (gas/oil) advanced-class combustion turbine generators with SCR and oxidation catalyst (TCEQ permit 178462); ~440 MW per unit implies H/J-class frames (OEM not published). SITE: BROWNFIELD - existing operating gas plant at 600 N Yucca Dr, Monahans, Ward County (existing 5x 65 MW CTs, gas supply and ERCOT interconnection in place); acreage not published. OWNERSHIP/STATUS: Permian Power I LLC (Vistra). FID Sep 29, 2025; $583M Texas Energy Fund loan Jun 2026 ($172M drawn by Jun 30, 2026); COD May/Jun 2028. EPC not public. INVESTMENT: Total project investment Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026); est. W&amp;C value $3,520,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://gov.texas.gov/news/post/governor-abbott-announces-texas-energy-fund-loan-for-860-mw-of-new-power-in-west-texas | https://investor.vistracorp.com/2025-09-29-Vistra-Announces-Plans-to-Build-New-Gas-Fueled-Dispatchable-Power-Units-in-the-Permian-Basin | https://www.gem.wiki/Permian_Power_power_station | https://www.tceq.texas.gov/downloads/permitting/air/bilingual/pending-permit-notices/178462-pls-english.pdf</t>
         </is>
       </c>
       <c r="CJ9" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $3,520,000 ($8/kW x 440 MW). Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026).</t>
+          <t>*RPBD* Total project investment: Not disclosed; financed in part by $583M Texas Energy Fund loan (3.0%, Jun 2026). Est. W&amp;C value: $3,520,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -15732,7 +15732,7 @@
       <c r="CF10" s="39" t="n"/>
       <c r="CG10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="CH10" s="38" t="inlineStr">
@@ -15742,12 +15742,12 @@
       </c>
       <c r="CI10" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018823691). Total project investment: Not public; PSC staff ~$1B for 3 units. W&amp;C value (est. $8/kW): $3,862,400. OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
+          <t>*RPBD* OVERVIEW: Georgia Power's first new gas turbines in a decade - three simple-cycle PEAKING units (~1,300 MW total, ~442-463 MW each) at Plant Yates; this record is Unit 9 (COD Q2 2027). Unit 8 Q4 2026, Unit 10 Q3 2027. ~600 construction jobs. Driven by Georgia load growth (data centers/industrial). TECHNOLOGY &amp; EQUIPMENT: 3x Mitsubishi Power M501JAC air-cooled combustion turbines with Mitsubishi Electric VP-X generators (assembled in Savannah, GA); dual-fuel gas/oil; ~30-minute start; hydrogen-capable with modifications. SITE: BROWNFIELD - existing Plant Yates generating site (former coal/gas station on the Chattahoochee River), Newnan, Coweta County, with existing transmission yard. OWNERSHIP/EPC: Georgia Power (Southern Company); EPC consortium Mitsubishi Power Americas + Black &amp; Veatch Construction (contract Jan 12, 2024). Cost not public (PSC staff ~$1B for 3 units). GA PSC monitoring docket 55931. INVESTMENT: Total project investment Not public; PSC staff ~$1B for 3 units; est. W&amp;C value $3,862,400 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Window: bulk cable for all 3 units most likely purchased 2024-25; remaining top-ups, change orders, spares. Ref: https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html | https://www.energy.gov/sites/default/files/2026-07/20260622_EnvReview_Completion_Yates.pdf | https://www.modernpowersystems.com/news/progress-at-1-3-gw-plant-yates-gas-fired-plant/</t>
         </is>
       </c>
       <c r="CJ10" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $3,862,400 ($8/kW x 482.8 MW). Total project investment: Not public; PSC staff ~$1B for 3 units.</t>
+          <t>*RPBD* Total project investment: Not public; PSC staff ~$1B for 3 units. Est. W&amp;C value: $3,862,400 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16024,7 @@
       <c r="CF11" s="39" t="n"/>
       <c r="CG11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*RPBD* CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="CH11" s="38" t="inlineStr">
@@ -16034,12 +16034,12 @@
       </c>
       <c r="CI11" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019705142). Total project investment: Not disclosed (GAJA rider). W&amp;C value (est. $8/kW): $3,568,000. OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
+          <t>*RPBD* OVERVIEW: 446 MW natural-gas SIMPLE-CYCLE combustion turbine (Entergy Arkansas 'Next Generation Arkansas'), replacing the 50+ year-old Lake Catherine Unit 4 (retiring end-2027). Formerly 'Lake Catherine 5'. ~260 peak construction jobs; Entergy prioritizing Arkansas contractors (vendor fair Mar 18, 2026). TECHNOLOGY &amp; EQUIPMENT: single advanced-class combustion turbine generator, hydrogen-capable (30% co-fire, future 100% conversion); Mitsubishi implied by the TSL/Mitsubishi Entergy program. SITE: BROWNFIELD - ~20 acres within the existing Lake Catherine Power Generation site, Jones Mill near Malvern, Hot Spring County; reuses existing gas, water and transmission infrastructure. OWNERSHIP/EPC: Entergy Arkansas; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). APSC CCN approved Apr 2025; site construction Q2 2026-Q2 2028; groundbreaking Aug 20, 2026; COD Q4 2028. Cost recovered via GAJA rider (not disclosed). INVESTMENT: Total project investment Not disclosed (GAJA rider); est. W&amp;C value $3,568,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Ref: https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station | https://www.modernpowersystems.com/news/entergy-arkansas-starts-construction-on-446-mw-ironwood-power-station/ | https://www.entergy.com/news/ironwood-power-plant-vendor-fair-for-arkansas-contractors-announced</t>
         </is>
       </c>
       <c r="CJ11" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $3,568,000 ($8/kW x 446 MW). Total project investment: Not disclosed (GAJA rider).</t>
+          <t>*RPBD* Total project investment: Not disclosed (GAJA rider). Est. W&amp;C value: $3,568,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -16328,7 +16328,7 @@
       <c r="CF12" s="39" t="n"/>
       <c r="CG12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*RPBD* CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="CH12" s="38" t="inlineStr">
@@ -16338,12 +16338,12 @@
       </c>
       <c r="CI12" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10017400436). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). W&amp;C value (est. $8/kW): $10,880,000. OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
+          <t>*RPBD* OVERVIEW: 1,360 MW natural-gas COMBINED-CYCLE block (first of two identical blocks, 2,720 MW total) at Duke's 'Person County Energy Complex' (Roxboro plant), enabling retirement of Roxboro coal units 1 &amp; 4. NCEMC co-owns ~225 MW. Nearby Microsoft-owned Person County Mega Park (~1,350 acres). TECHNOLOGY &amp; EQUIPMENT: 2x1 advanced-class, hydrogen-capable CC - 2x GE Vernova gas turbines, 2x HRSGs, 1x GE Vernova steam turbine generator (~450 tons); first GT on site Jul 23, 2026. SITE: BROWNFIELD - ~50 acres of undeveloped land within the existing Roxboro coal plant property, Semora Road side, Semora/Roxboro, Person County. OWNERSHIP/EPC: Duke Energy Progress (majority) + NCEMC; full EPC Zachry Group (awarded Aug 2025). NCUC CPCN Oct 2025; groundbreaking Feb 13, 2026; COD Q4 2028 (CC2 Q4 2029). Cost ~$2.13B (CC1). Two new tie lines from the site. INVESTMENT: Total project investment ~$2.13B (CC1, DEP Class 3 estimate); est. W&amp;C value $10,880,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. CC2 doubles the scope ~1 year later with the same EPC. Ref: https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html | https://www.duke-energy.com/info/person | https://www.theassemblync.com/news/business/person-county-microsoft-data-center-nondisclosure-agreements/</t>
         </is>
       </c>
       <c r="CJ12" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $10,880,000 ($8/kW x 1,360 MW). Total project investment: ~$2.13B (CC1, DEP Class 3 estimate).</t>
+          <t>*RPBD* Total project investment: ~$2.13B (CC1, DEP Class 3 estimate). Est. W&amp;C value: $10,880,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -16634,7 +16634,7 @@
       <c r="CF13" s="39" t="n"/>
       <c r="CG13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
+          <t>*RPBD* MAIN WINDOW LIKELY PASSED: HRSG erection May 2026 ("anchor bolts up"), COD May 2028 -&gt; bulk cable likely bought; remaining late releases, change orders, I&amp;C top-ups. EPC TSL Power Partners (Kiewit/TIC), Kiewit 200+ on site. Use as entry to TSL Entergy program buy for sister plants. Yes Energy 879 MW/$651M vs Entergy 754 MW/$1.2B.</t>
         </is>
       </c>
       <c r="CH13" s="38" t="inlineStr">
@@ -16644,12 +16644,12 @@
       </c>
       <c r="CI13" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10018299981). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="CJ13" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $6,032,000 ($8/kW x 754 MW). Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed.</t>
+          <t>*RPBD* Total project investment: ~$1.2B (Entergy); Yes Energy $651M not confirmed. Est. W&amp;C value: $6,032,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -16926,7 +16926,7 @@
       <c r="CF14" s="39" t="n"/>
       <c r="CG14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
+          <t>*RPBD* URGENT: groundbreaking Oct 21 2025, Baxter Wilson demolition Dec 2025, COD Aug 2028 -&gt; cable window now through ~Feb 2027; may be partly placed if TSL bought with Delta Blues. Linked contextually to AWS $3B Vicksburg campus. Entergy MS media line 769-262-0745.</t>
         </is>
       </c>
       <c r="CH14" s="38" t="inlineStr">
@@ -16936,12 +16936,12 @@
       </c>
       <c r="CI14" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019088992). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. W&amp;C value (est. $8/kW): $6,032,000. OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant, next phase of 'Superpower Mississippi'; ~560 construction jobs, 21 permanent. Contextually linked to Amazon/AWS's $3B Vicksburg data-center campus (AWS covers its service-extension costs). TECHNOLOGY &amp; EQUIPMENT: combined cycle (gas turbine + HRSG + steam turbine), hydrogen-blend capable and carbon-capture enabled; turbine OEM not confirmed (Mitsubishi likely via TSL/Mitsubishi Entergy program). SITE: BROWNFIELD - former Baxter Wilson Steam Electric Station (1960s gas/oil plant, retired 2022; large structures demolished Dec 17, 2025), 770 Kemp Bottom Rd, Vicksburg, Warren County, on the Mississippi River; existing transmission/gas corridors (acreage not published). OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power Americas (per TIC Entergy Program page). Groundbreaking Oct 21, 2025; COD Aug 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $700M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Ref: https://www.entergymississippi.com/generation/vicksburg | https://www.powermag.com/entergy-mississippi-adding-third-gas-fired-power-plant-to-superpower-strategy/ | https://www.datacenterdynamics.com/en/news/amazon-to-build-3bn-data-center-campus-in-vicksburg-mississippi/</t>
         </is>
       </c>
       <c r="CJ14" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $6,032,000 ($8/kW x 754 MW). Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed.</t>
+          <t>*RPBD* Total project investment: ~$1.2B (Entergy); Yes Energy $700M not confirmed. Est. W&amp;C value: $6,032,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -17220,7 +17220,7 @@
       <c r="CF15" s="39" t="n"/>
       <c r="CG15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*RPBD* CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="CH15" s="38" t="inlineStr">
@@ -17230,12 +17230,12 @@
       </c>
       <c r="CI15" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019254864). Total project investment: ~$500M capital investment (Invenergy). W&amp;C value (est. $8/kW): $7,344,000. OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
+          <t>*RPBD* OVERVIEW: ~918-935 MW natural-gas SIMPLE-CYCLE PEAKING plant developed by Invenergy and to be acquired by Indiana Michigan Power (AEP) at COD (Mar 31, 2029) to meet data-center-driven load growth (AWS, Google, Microsoft). Formerly queued as Sullivan Generating Station 1 &amp; 2 (1,150 MW CC concept). TECHNOLOGY &amp; EQUIPMENT: 4x GE Vernova 7F.05 combustion turbines (~232 MW each), dual-fuel natural gas with ultra-low-sulfur distillate backup; gas via ~5.5-mile 24-inch ONEOK lateral. SITE: BROWNFIELD-ADJACENT - next to I&amp;M's retired, demolished Breed coal plant, CR 925N, Fairbanks Township, Sullivan County; ~64-acre plant footprint within ~356-acre parcel (local meeting summary - verify). Invenergy holds land under purchase option. INTERCONNECTION: AEP/I&amp;M Sullivan 345 kV station (new 345 kV breakers), PJM. OWNERSHIP/STATUS: Invenergy (developer) -&gt; I&amp;M; IURC Cause 46389 order expected end-2026; constructor The Boldt Company lists construction Sep 2026-Feb 2029; ~$500M capital (Invenergy). INVESTMENT: Total project investment ~$500M capital investment (Invenergy); est. W&amp;C value $7,344,000 ($8/kW). W&amp;C NEEDS (simple-cycle peaker): MV power cable (5-35 kV) for auxiliary transformers, MV switchgear, fuel-gas compressors and black-start/aux systems; 600V power &amp; TC-ER tray cable for turbine packages, MCCs, fuel oil forwarding (if dual fuel) and SCR/ammonia systems; shielded instrumentation &amp; control cable; bare copper grounding grid per unit and switchyard; switchyard control/relay cable; building wire for control/admin buildings. Less cable per MW than a CC (no HRSG/steam cycle). Dual-fuel adds fuel-oil system cabling. Ref: https://www.aep.com/news/stories/view/11850/ | https://sycamoreriverside.invenergy.com/about-project | https://www.pjm.com/pub/planning/project-queues/facilities/ab1087_fac.pdf | https://www.gem.wiki/Sycamore_Riverside_Energy_Center</t>
         </is>
       </c>
       <c r="CJ15" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $7,344,000 ($8/kW x 918 MW). Total project investment: ~$500M capital investment (Invenergy).</t>
+          <t>*RPBD* Total project investment: ~$500M capital investment (Invenergy). Est. W&amp;C value: $7,344,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -17514,7 +17514,7 @@
       <c r="CF16" s="39" t="n"/>
       <c r="CG16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*RPBD* CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="CH16" s="38" t="inlineStr">
@@ -17524,12 +17524,12 @@
       </c>
       <c r="CI16" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019228423). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). W&amp;C value (est. $8/kW): $12,000,000. OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*RPBD* OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,000,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="CJ16" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $12,000,000 ($8/kW x 1,500 MW). Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony).</t>
+          <t>*RPBD* Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). Est. W&amp;C value: $12,000,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -17818,7 +17818,7 @@
       <c r="CF17" s="39" t="n"/>
       <c r="CG17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*RPBD* CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="CH17" s="38" t="inlineStr">
@@ -17828,12 +17828,12 @@
       </c>
       <c r="CI17" s="38" t="inlineStr">
         <is>
-          <t>*Reported Pipeline/BD selection - Source: Yes Energy Generation Projects 08/24/2026, W&amp;C-Filtered Selection (Project ID 10019089005). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. W&amp;C value (est. $8/kW): $6,560,000. OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+          <t>*RPBD* OVERVIEW: ~754-820 MW natural-gas COMBINED-CYCLE unit approved with Franklin Farms to support Meta's Hyperion load; paired with proposed Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16, 2026) - ~$3.75B WF5+6 program, 700+ construction jobs 2026-2030. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine, HRSG, steam turbine (EIA: 2 generators, 820 MW nameplate). SITE: BROWNFIELD - existing Entergy Waterford generating complex at Killona/Taft, St. Charles Parish, on the Mississippi River (home to Waterford 1 &amp; 2 gas/oil units and Waterford 3 nuclear); soft soils require ~100,000 truckloads of surcharge fill (site prep since Nov 2025). INTERCONNECTION: Waterford 500 kV substation via ~0.25-mile 500 kV gen-tie (MISO E0029). OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC + Sargent &amp; Lundy) per LPSC Waterford 6 filing. Main construction late 2026; COD 2029. Cost ~ $1.2B implied. INVESTMENT: Total project investment ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed; est. W&amp;C value $6,560,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus 500 kV gen-tie; bundle Waterford 5 + 6 as one cable package. Ref: https://www.entergylouisiana.com/waterford5-6 | https://www.interconnection.fyi/project/miso-e0029 | https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
         </is>
       </c>
       <c r="CJ17" s="38" t="inlineStr">
         <is>
-          <t>Source: Yes Energy Generation Projects 08/24/2026 (filtered: NG, Adv. Dev./Under Construction, COD 2027-2030, prob &gt;=0.7), verified by web research 10/29/2026. Est. W&amp;C value $6,560,000 ($8/kW x 820 MW). Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed.</t>
+          <t>*RPBD* Total project investment: ~$1.2B implied (similar to each Franklin Farms unit); Yes Energy $1.75B not confirmed. Est. W&amp;C value: $6,560,000 ($8/kW).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge verified contact routes, verification tab and fixes from review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Sources" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Named Contacts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="ProjectStage">'Dropdowns'!$A$7:INDEX('Dropdowns'!$A$7:$A$106,COUNTA('Dropdowns'!$A$7:$A$106))</definedName>
@@ -49,7 +50,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -91,6 +92,10 @@
       <color theme="10"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -143,7 +148,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -305,6 +310,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0"/>
@@ -1975,8 +1981,9 @@
         </is>
       </c>
       <c r="L7" s="40" t="n"/>
-      <c r="M7" s="41" t="n">
-        <v>9624000</v>
+      <c r="M7" s="41">
+        <f>P7*1000*8</f>
+        <v/>
       </c>
       <c r="N7" s="42" t="n"/>
       <c r="O7" s="43" t="n"/>
@@ -2154,8 +2161,9 @@
         </is>
       </c>
       <c r="L8" s="40" t="n"/>
-      <c r="M8" s="41" t="n">
-        <v>9720000</v>
+      <c r="M8" s="41">
+        <f>P8*1000*8</f>
+        <v/>
       </c>
       <c r="N8" s="42" t="n"/>
       <c r="O8" s="43" t="n"/>
@@ -2321,8 +2329,9 @@
         </is>
       </c>
       <c r="L9" s="40" t="n"/>
-      <c r="M9" s="41" t="n">
-        <v>3520000</v>
+      <c r="M9" s="41">
+        <f>P9*1000*8</f>
+        <v/>
       </c>
       <c r="N9" s="42" t="n"/>
       <c r="O9" s="43" t="n"/>
@@ -2488,8 +2497,9 @@
         </is>
       </c>
       <c r="L10" s="40" t="n"/>
-      <c r="M10" s="41" t="n">
-        <v>3862400</v>
+      <c r="M10" s="41">
+        <f>P10*1000*8</f>
+        <v/>
       </c>
       <c r="N10" s="42" t="n"/>
       <c r="O10" s="43" t="n"/>
@@ -2655,8 +2665,9 @@
         </is>
       </c>
       <c r="L11" s="40" t="n"/>
-      <c r="M11" s="41" t="n">
-        <v>3568000</v>
+      <c r="M11" s="41">
+        <f>P11*1000*8</f>
+        <v/>
       </c>
       <c r="N11" s="42" t="n"/>
       <c r="O11" s="43" t="n"/>
@@ -2822,8 +2833,9 @@
         </is>
       </c>
       <c r="L12" s="40" t="n"/>
-      <c r="M12" s="41" t="n">
-        <v>10880000</v>
+      <c r="M12" s="41">
+        <f>P12*1000*8</f>
+        <v/>
       </c>
       <c r="N12" s="42" t="n"/>
       <c r="O12" s="43" t="n"/>
@@ -2997,8 +3009,9 @@
         </is>
       </c>
       <c r="L13" s="40" t="n"/>
-      <c r="M13" s="41" t="n">
-        <v>6032000</v>
+      <c r="M13" s="41">
+        <f>P13*1000*8</f>
+        <v/>
       </c>
       <c r="N13" s="42" t="n"/>
       <c r="O13" s="43" t="n"/>
@@ -3096,7 +3109,7 @@
       </c>
       <c r="AL13" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the aging Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="AM13" s="40" t="n"/>
@@ -3153,7 +3166,7 @@
       </c>
       <c r="F14" s="38" t="inlineStr">
         <is>
-          <t>Ernest Rufus, Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
+          <t>Ernest Rufus, Senior Manager, Capital Projects (Vicksburg role to confirm)</t>
         </is>
       </c>
       <c r="G14" s="36" t="inlineStr">
@@ -3174,8 +3187,9 @@
         </is>
       </c>
       <c r="L14" s="40" t="n"/>
-      <c r="M14" s="41" t="n">
-        <v>6032000</v>
+      <c r="M14" s="41">
+        <f>P14*1000*8</f>
+        <v/>
       </c>
       <c r="N14" s="42" t="n"/>
       <c r="O14" s="43" t="n"/>
@@ -3268,7 +3282,7 @@
       </c>
       <c r="AK14" s="38" t="inlineStr">
         <is>
-          <t>Engage TSL/TIC procurement and Ernest Rufus immediately.</t>
+          <t>Engage TSL/TIC procurement now; confirm Ernest Rufus covers Vicksburg (confirmed on Delta Blues only) and ask for the named project buyer.</t>
         </is>
       </c>
       <c r="AL14" s="38" t="inlineStr">
@@ -3341,8 +3355,9 @@
         </is>
       </c>
       <c r="L15" s="40" t="n"/>
-      <c r="M15" s="41" t="n">
-        <v>7344000</v>
+      <c r="M15" s="41">
+        <f>P15*1000*8</f>
+        <v/>
       </c>
       <c r="N15" s="42" t="n"/>
       <c r="O15" s="43" t="n"/>
@@ -3510,13 +3525,14 @@
         </is>
       </c>
       <c r="L16" s="40" t="n"/>
-      <c r="M16" s="41" t="n">
-        <v>12000000</v>
+      <c r="M16" s="41">
+        <f>P16*1000*8</f>
+        <v/>
       </c>
       <c r="N16" s="42" t="n"/>
       <c r="O16" s="43" t="n"/>
       <c r="P16" s="44" t="n">
-        <v>1500</v>
+        <v>1508</v>
       </c>
       <c r="Q16" s="44" t="n">
         <v>500</v>
@@ -3611,7 +3627,7 @@
       </c>
       <c r="AL16" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,000,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*RPBD* OVERVIEW: ~1,508 MW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,064,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="AM16" s="40" t="n"/>
@@ -3679,8 +3695,9 @@
         </is>
       </c>
       <c r="L17" s="40" t="n"/>
-      <c r="M17" s="41" t="n">
-        <v>6560000</v>
+      <c r="M17" s="41">
+        <f>P17*1000*8</f>
+        <v/>
       </c>
       <c r="N17" s="42" t="n"/>
       <c r="O17" s="43" t="n"/>
@@ -14622,9 +14639,17 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="K7" s="39" t="n"/>
+      <c r="K7" s="36" t="inlineStr">
+        <is>
+          <t>+1 312-582-1094</t>
+        </is>
+      </c>
       <c r="L7" s="39" t="n"/>
-      <c r="M7" s="39" t="n"/>
+      <c r="M7" s="36" t="inlineStr">
+        <is>
+          <t>dbirmingham@invenergy.com</t>
+        </is>
+      </c>
       <c r="N7" s="39" t="n"/>
       <c r="O7" s="37" t="inlineStr">
         <is>
@@ -14670,8 +14695,9 @@
           <t>IPP</t>
         </is>
       </c>
-      <c r="AI7" s="49" t="n">
-        <v>9624000</v>
+      <c r="AI7" s="49">
+        <f>AL7*1000*8</f>
+        <v/>
       </c>
       <c r="AJ7" s="50" t="n"/>
       <c r="AK7" s="45" t="n">
@@ -14970,8 +14996,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI8" s="49" t="n">
-        <v>9720000</v>
+      <c r="AI8" s="49">
+        <f>AL8*1000*8</f>
+        <v/>
       </c>
       <c r="AJ8" s="50" t="n"/>
       <c r="AK8" s="45" t="n">
@@ -15262,8 +15289,9 @@
           <t>IPP</t>
         </is>
       </c>
-      <c r="AI9" s="49" t="n">
-        <v>3520000</v>
+      <c r="AI9" s="49">
+        <f>AL9*1000*8</f>
+        <v/>
       </c>
       <c r="AJ9" s="50" t="n"/>
       <c r="AK9" s="45" t="n">
@@ -15550,8 +15578,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI10" s="49" t="n">
-        <v>3862400</v>
+      <c r="AI10" s="49">
+        <f>AL10*1000*8</f>
+        <v/>
       </c>
       <c r="AJ10" s="50" t="n"/>
       <c r="AK10" s="45" t="n">
@@ -15846,8 +15875,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI11" s="49" t="n">
-        <v>3568000</v>
+      <c r="AI11" s="49">
+        <f>AL11*1000*8</f>
+        <v/>
       </c>
       <c r="AJ11" s="50" t="n"/>
       <c r="AK11" s="45" t="n">
@@ -16138,8 +16168,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI12" s="49" t="n">
-        <v>10880000</v>
+      <c r="AI12" s="49">
+        <f>AL12*1000*8</f>
+        <v/>
       </c>
       <c r="AJ12" s="50" t="n"/>
       <c r="AK12" s="45" t="n">
@@ -16442,8 +16473,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI13" s="49" t="n">
-        <v>6032000</v>
+      <c r="AI13" s="49">
+        <f>AL13*1000*8</f>
+        <v/>
       </c>
       <c r="AJ13" s="50" t="n"/>
       <c r="AK13" s="45" t="n">
@@ -16644,7 +16676,7 @@
       </c>
       <c r="CI13" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the 1950s-era Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
+          <t>*RPBD* OVERVIEW: 754 MW natural-gas COMBINED-CYCLE plant ('Superpower Mississippi'), replacing the aging Gerald Andrus Steam Electric Station; serves ~385,000 homes across Entergy Mississippi's 45 counties. TECHNOLOGY &amp; EQUIPMENT: 1x1 combined cycle - Mitsubishi Power M501JAC gas turbine (per GEM), HRSG (modules being lifted May 2026), steam turbine; dual-fuel, hydrogen-blend capable. SITE: BROWNFIELD-ADJACENT - new footprint within ~1 mile of the Andrus plant, 85 Stokes King Road, Greenville, Washington County; reuses Andrus transmission and gas infrastructure (acreage not published). INTERCONNECTION: ~1.5 miles of new transmission line to the existing substation next to Andrus; new Delta Blues substation. OWNERSHIP/EPC: Entergy Mississippi; EPC TSL Power Partners (Kiewit Power Constructors / TIC; Kiewit 200+ on site). Groundbreaking Nov 2024; COD May 2028; ~$1.2B. INVESTMENT: Total project investment ~$1.2B (Entergy); Yes Energy $651M not confirmed; est. W&amp;C value $6,032,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Plus ~1.5 mi transmission line conductor and substation cable. Status: above-ground erection since May 2026 - bulk cable likely ordered. Ref: https://www.power-eng.com/gas/combined-cycle/entergy-mississippi-breaks-ground-on-754-mw-combined-cycle-plant/ | https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction | https://www.gem.wiki/Delta_Blues_Advanced_Power_Station | https://opcgis.deq.state.ms.us/ensearchonline/ai_info.aspx?ai=86260</t>
         </is>
       </c>
       <c r="CJ13" s="38" t="inlineStr">
@@ -16687,7 +16719,7 @@
       <c r="G14" s="40" t="n"/>
       <c r="H14" s="38" t="inlineStr">
         <is>
-          <t>Senior Manager, Capital Projects (Delta Blues &amp; Vicksburg)</t>
+          <t>Senior Manager, Capital Projects (Vicksburg role to confirm)</t>
         </is>
       </c>
       <c r="I14" s="37" t="inlineStr">
@@ -16748,8 +16780,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI14" s="49" t="n">
-        <v>6032000</v>
+      <c r="AI14" s="49">
+        <f>AL14*1000*8</f>
+        <v/>
       </c>
       <c r="AJ14" s="50" t="n"/>
       <c r="AK14" s="45" t="n">
@@ -16931,7 +16964,7 @@
       </c>
       <c r="CH14" s="38" t="inlineStr">
         <is>
-          <t>Engage TSL/TIC procurement and Ernest Rufus immediately.</t>
+          <t>Engage TSL/TIC procurement now; confirm Ernest Rufus covers Vicksburg (confirmed on Delta Blues only) and ask for the named project buyer.</t>
         </is>
       </c>
       <c r="CI14" s="38" t="inlineStr">
@@ -17040,8 +17073,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI15" s="49" t="n">
-        <v>7344000</v>
+      <c r="AI15" s="49">
+        <f>AL15*1000*8</f>
+        <v/>
       </c>
       <c r="AJ15" s="50" t="n"/>
       <c r="AK15" s="45" t="n">
@@ -17334,15 +17368,16 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI16" s="49" t="n">
-        <v>12000000</v>
+      <c r="AI16" s="49">
+        <f>AL16*1000*8</f>
+        <v/>
       </c>
       <c r="AJ16" s="50" t="n"/>
       <c r="AK16" s="45" t="n">
         <v>47088</v>
       </c>
       <c r="AL16" s="44" t="n">
-        <v>1500</v>
+        <v>1508</v>
       </c>
       <c r="AM16" s="44" t="n">
         <v>500</v>
@@ -17524,12 +17559,12 @@
       </c>
       <c r="CI16" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* OVERVIEW: ~1.5 GW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,000,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
+          <t>*RPBD* OVERVIEW: ~1,508 MW natural-gas COMBINED-CYCLE station (two units) built to power Meta's Hyperion AI data-center campus; Meta pays the plants' full revenue requirement for 15 years. Air permit name 'Titanium Advanced Power Station'. ~7 more Hyperion plants (~5.2 GW) proposed, LPSC vote Dec 2026. TECHNOLOGY &amp; EQUIPMENT: 2x 1x1 combined-cycle blocks - Mitsubishi Power M501JAC gas turbines, HRSGs, steam turbines (~754-780 MW each); hydrogen-capable (30% co-fire), carbon-capture ready; IMI valve package (Sep 2026). SITE: GREENFIELD - former agricultural land on the state-owned Franklin Farms megasite (~1,400-2,250 acres total incl. Meta campus) along LA Hwy 183 near Holly Ridge, Richland Parish. INTERCONNECTION: Entergy 500 kV system - ~100 miles of new 500 kV lines (~$1.2B), eight new 230 kV lines, Sterlington 500 kV upgrades. OWNERSHIP/EPC: Entergy Louisiana; EPC TSL Power Partners (TIC/Kiewit + Sargent &amp; Lundy) with Mitsubishi Power. LPSC approval Aug 2025; groundbreaking Dec 1, 2025; COD Dec 2028; ~$2.39B for both units. INVESTMENT: Total project investment ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony); est. W&amp;C value $12,064,000 ($8/kW). W&amp;C NEEDS (combined cycle): MV power cable (5-35 kV) from unit auxiliary/station service transformers to plant MV switchgear and large motors (boiler feed pumps, condensate &amp; circulating water pumps, cooling tower/ACC fans, gas compressors); 600V power &amp; TC-ER tray cable for MCCs, HRSG/steam-turbine auxiliaries, BOP and water treatment; shielded instrumentation &amp; control cable (DCS, turbine controls, CEMS); bare copper grounding grid; switchyard control/relay cable; lighting, building wire and fire-alarm in admin/warehouse/control buildings. Separate opportunity: HV/500 kV transmission conductor and substation cable. Ref: https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation | https://www.ticus.com/entergy-program/ | https://www.gem.wiki/Franklin_Farms_power_station | https://www.datacenterdynamics.com/en/news/entergy-breaks-ground-on-two-natural-gas-plants-for-metas-2gw-data-center-in-richland-parish-louisiana/</t>
         </is>
       </c>
       <c r="CJ16" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). Est. W&amp;C value: $12,000,000 ($8/kW).</t>
+          <t>*RPBD* Total project investment: ~$2.39B (Franklin Farms 1 &amp; 2, LPSC testimony). Est. W&amp;C value: $12,064,000 ($8/kW).</t>
         </is>
       </c>
     </row>
@@ -17628,8 +17663,9 @@
           <t>IOU</t>
         </is>
       </c>
-      <c r="AI17" s="49" t="n">
-        <v>6560000</v>
+      <c r="AI17" s="49">
+        <f>AL17*1000*8</f>
+        <v/>
       </c>
       <c r="AJ17" s="50" t="n"/>
       <c r="AK17" s="45" t="n">
@@ -35723,7 +35759,7 @@
       </c>
       <c r="C46" s="52" t="inlineStr">
         <is>
-          <t>MV power cable: 42% of W&amp;C = $5,040,000</t>
+          <t>MV power cable: 42% of W&amp;C = $5,066,880</t>
         </is>
       </c>
     </row>
@@ -35740,7 +35776,7 @@
       </c>
       <c r="C47" s="52" t="inlineStr">
         <is>
-          <t>Tray cable (TC) - control &amp; instrumentation: 43% of W&amp;C = $5,160,000</t>
+          <t>Tray cable (TC) - control &amp; instrumentation: 43% of W&amp;C = $5,187,520</t>
         </is>
       </c>
     </row>
@@ -35757,7 +35793,7 @@
       </c>
       <c r="C48" s="52" t="inlineStr">
         <is>
-          <t>PV / LV single-conductor power: 10% of W&amp;C = $1,200,000</t>
+          <t>PV / LV single-conductor power: 10% of W&amp;C = $1,206,400</t>
         </is>
       </c>
     </row>
@@ -35774,7 +35810,7 @@
       </c>
       <c r="C49" s="52" t="inlineStr">
         <is>
-          <t>Other - substation / switchyard: 5% of W&amp;C = $600,000</t>
+          <t>Other - substation / switchyard: 5% of W&amp;C = $603,200</t>
         </is>
       </c>
     </row>
@@ -44335,7 +44371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -44807,6 +44843,210 @@
       <c r="B39" s="55" t="inlineStr">
         <is>
           <t>https://www.entergy.com/blog/the-dirt-on-dirt-from-digging-soil-to-boosting-louisianas-economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B40" s="55" t="inlineStr">
+        <is>
+          <t>https://forestjunctionenergycenter.invenergy.com/news-and-resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B41" s="55" t="inlineStr">
+        <is>
+          <t>https://apps.dnr.wi.gov/warp_ext/am_permittracking2.aspx?id=38822</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B42" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-texas-orange-county-advanced-power-station-begins-delivering-reliable-power-to-southeast-texas</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B43" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B44" s="55" t="inlineStr">
+        <is>
+          <t>https://hub.vistracorp.com/vistra-announces-plans-to-build-new-dispatchable-generation-in-texas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B45" s="55" t="inlineStr">
+        <is>
+          <t>https://vistracorp.com/supply-chain/how-do-we-source/ | https://vistracorp.com/supply-chain/faq/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B46" s="55" t="inlineStr">
+        <is>
+          <t>https://www.southerncompany.com/contact-us.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B47" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B48" s="55" t="inlineStr">
+        <is>
+          <t>https://s201.q4cdn.com/714390239/files/doc_presentations/2026/Jun/09/Entergy-2026-Investor-Day.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B49" s="55" t="inlineStr">
+        <is>
+          <t>https://zachrygroup.com/procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B50" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Vicksburg Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B51" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B52" s="55" t="inlineStr">
+        <is>
+          <t>https://sycamoreriverside.invenergy.com/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B53" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B54" s="55" t="inlineStr">
+        <is>
+          <t>https://s201.q4cdn.com/714390239/files/doc_presentations/2026/Jun/09/Entergy-2026-Investor-Day.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B55" s="55" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B56" s="55" t="inlineStr">
+        <is>
+          <t>https://s201.q4cdn.com/714390239/files/doc_presentations/2026/Jun/09/Entergy-2026-Investor-Day.pdf</t>
         </is>
       </c>
     </row>
@@ -44850,6 +45090,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -44861,7 +45118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -44872,6 +45129,11 @@
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44915,6 +45177,31 @@
           <t>Confidence</t>
         </is>
       </c>
+      <c r="I1" s="53" t="inlineStr">
+        <is>
+          <t>Verified email</t>
+        </is>
+      </c>
+      <c r="J1" s="53" t="inlineStr">
+        <is>
+          <t>Verified phone</t>
+        </is>
+      </c>
+      <c r="K1" s="53" t="inlineStr">
+        <is>
+          <t>Contact note</t>
+        </is>
+      </c>
+      <c r="L1" s="53" t="inlineStr">
+        <is>
+          <t>Contact source</t>
+        </is>
+      </c>
+      <c r="M1" s="53" t="inlineStr">
+        <is>
+          <t>Checked on</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="54" t="inlineStr">
@@ -44953,6 +45240,31 @@
           <t>News quote</t>
         </is>
       </c>
+      <c r="I2" s="54" t="inlineStr">
+        <is>
+          <t>dbirmingham@invenergy.com</t>
+        </is>
+      </c>
+      <c r="J2" s="54" t="inlineStr">
+        <is>
+          <t>+1 312-582-1094</t>
+        </is>
+      </c>
+      <c r="K2" s="54" t="inlineStr">
+        <is>
+          <t>Published business contact; cross-project DNR record. Forest Junction role listed by developer.</t>
+        </is>
+      </c>
+      <c r="L2" s="56" t="inlineStr">
+        <is>
+          <t>https://apps.dnr.wi.gov/warp_ext/am_permittracking2.aspx?id=38822</t>
+        </is>
+      </c>
+      <c r="M2" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="54" t="inlineStr">
@@ -44991,6 +45303,19 @@
           <t>News quote</t>
         </is>
       </c>
+      <c r="I3" s="54" t="n"/>
+      <c r="J3" s="54" t="n"/>
+      <c r="K3" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L3" s="54" t="n"/>
+      <c r="M3" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="54" t="inlineStr">
@@ -45029,6 +45354,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I4" s="54" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L4" s="54" t="n"/>
+      <c r="M4" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="54" t="inlineStr">
@@ -45067,6 +45405,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I5" s="54" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L5" s="54" t="n"/>
+      <c r="M5" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="54" t="inlineStr">
@@ -45105,6 +45456,19 @@
           <t>Company website</t>
         </is>
       </c>
+      <c r="I6" s="54" t="n"/>
+      <c r="J6" s="54" t="n"/>
+      <c r="K6" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L6" s="54" t="n"/>
+      <c r="M6" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="54" t="inlineStr">
@@ -45147,6 +45511,19 @@
           <t>Official website</t>
         </is>
       </c>
+      <c r="I7" s="54" t="n"/>
+      <c r="J7" s="54" t="n"/>
+      <c r="K7" s="54" t="inlineStr">
+        <is>
+          <t>Original media line not independently reconfirmed; not a project procurement number.</t>
+        </is>
+      </c>
+      <c r="L7" s="54" t="n"/>
+      <c r="M7" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="54" t="inlineStr">
@@ -45185,6 +45562,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I8" s="54" t="n"/>
+      <c r="J8" s="54" t="n"/>
+      <c r="K8" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L8" s="54" t="n"/>
+      <c r="M8" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="54" t="inlineStr">
@@ -45223,6 +45613,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I9" s="54" t="n"/>
+      <c r="J9" s="54" t="n"/>
+      <c r="K9" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L9" s="54" t="n"/>
+      <c r="M9" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
@@ -45261,6 +45664,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I10" s="54" t="n"/>
+      <c r="J10" s="54" t="n"/>
+      <c r="K10" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L10" s="54" t="n"/>
+      <c r="M10" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
@@ -45299,6 +45715,19 @@
           <t>Company website - indirect</t>
         </is>
       </c>
+      <c r="I11" s="54" t="n"/>
+      <c r="J11" s="54" t="n"/>
+      <c r="K11" s="54" t="inlineStr">
+        <is>
+          <t>Original source concerns Plant Barry; Yates assignment NOT verified.</t>
+        </is>
+      </c>
+      <c r="L11" s="54" t="n"/>
+      <c r="M11" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
@@ -45337,6 +45766,19 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I12" s="54" t="n"/>
+      <c r="J12" s="54" t="n"/>
+      <c r="K12" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L12" s="54" t="n"/>
+      <c r="M12" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
@@ -45375,6 +45817,19 @@
           <t>News</t>
         </is>
       </c>
+      <c r="I13" s="54" t="n"/>
+      <c r="J13" s="54" t="n"/>
+      <c r="K13" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L13" s="54" t="n"/>
+      <c r="M13" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
@@ -45413,6 +45868,19 @@
           <t>Regulatory document</t>
         </is>
       </c>
+      <c r="I14" s="54" t="n"/>
+      <c r="J14" s="54" t="n"/>
+      <c r="K14" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L14" s="54" t="n"/>
+      <c r="M14" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="54" t="inlineStr">
@@ -45455,6 +45923,19 @@
           <t>Regulatory document</t>
         </is>
       </c>
+      <c r="I15" s="54" t="n"/>
+      <c r="J15" s="54" t="n"/>
+      <c r="K15" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L15" s="54" t="n"/>
+      <c r="M15" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="54" t="inlineStr">
@@ -45493,6 +45974,19 @@
           <t>Org website</t>
         </is>
       </c>
+      <c r="I16" s="54" t="n"/>
+      <c r="J16" s="54" t="n"/>
+      <c r="K16" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L16" s="54" t="n"/>
+      <c r="M16" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="54" t="inlineStr">
@@ -45531,6 +46025,19 @@
           <t>LinkedIn - verify</t>
         </is>
       </c>
+      <c r="I17" s="54" t="n"/>
+      <c r="J17" s="54" t="n"/>
+      <c r="K17" s="54" t="inlineStr">
+        <is>
+          <t>LinkedIn-derived suggestion; current procurement assignment not independently confirmed.</t>
+        </is>
+      </c>
+      <c r="L17" s="54" t="n"/>
+      <c r="M17" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="54" t="inlineStr">
@@ -45573,6 +46080,31 @@
           <t>Official website</t>
         </is>
       </c>
+      <c r="I18" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J18" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+      <c r="K18" s="54" t="inlineStr">
+        <is>
+          <t>Shared supplier support; not a project buyer.</t>
+        </is>
+      </c>
+      <c r="L18" s="56" t="inlineStr">
+        <is>
+          <t>https://supplier.entergy.com/psc/supprd/SUPPLIER/ERP/c/SCP_PUBLIC_MENU_FL.SCP_PUB_FAQ_CMP_FL.GBL</t>
+        </is>
+      </c>
+      <c r="M18" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
@@ -45611,6 +46143,19 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I19" s="54" t="n"/>
+      <c r="J19" s="54" t="n"/>
+      <c r="K19" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L19" s="54" t="n"/>
+      <c r="M19" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
@@ -45649,6 +46194,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I20" s="54" t="n"/>
+      <c r="J20" s="54" t="n"/>
+      <c r="K20" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L20" s="54" t="n"/>
+      <c r="M20" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="54" t="inlineStr">
@@ -45687,6 +46245,19 @@
           <t>News quote</t>
         </is>
       </c>
+      <c r="I21" s="54" t="n"/>
+      <c r="J21" s="54" t="n"/>
+      <c r="K21" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L21" s="54" t="n"/>
+      <c r="M21" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="54" t="inlineStr">
@@ -45725,6 +46296,19 @@
           <t>LinkedIn - verify</t>
         </is>
       </c>
+      <c r="I22" s="54" t="n"/>
+      <c r="J22" s="54" t="n"/>
+      <c r="K22" s="54" t="inlineStr">
+        <is>
+          <t>Talent acquisition is not a procurement contact; project purchasing role not confirmed.</t>
+        </is>
+      </c>
+      <c r="L22" s="54" t="n"/>
+      <c r="M22" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="54" t="inlineStr">
@@ -45763,6 +46347,19 @@
           <t>Official blog</t>
         </is>
       </c>
+      <c r="I23" s="54" t="n"/>
+      <c r="J23" s="54" t="n"/>
+      <c r="K23" s="54" t="inlineStr">
+        <is>
+          <t>Entergy confirms Ernest Rufus as senior manager, capital projects on Delta Blues; direct email/phone not found.</t>
+        </is>
+      </c>
+      <c r="L23" s="54" t="n"/>
+      <c r="M23" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="54" t="inlineStr">
@@ -45805,6 +46402,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I24" s="54" t="n"/>
+      <c r="J24" s="54" t="n"/>
+      <c r="K24" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L24" s="54" t="n"/>
+      <c r="M24" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="54" t="inlineStr">
@@ -45840,7 +46450,20 @@
       </c>
       <c r="H25" s="54" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>News - Vicksburg role to confirm (Entergy confirms Delta Blues only)</t>
+        </is>
+      </c>
+      <c r="I25" s="54" t="n"/>
+      <c r="J25" s="54" t="n"/>
+      <c r="K25" s="54" t="inlineStr">
+        <is>
+          <t>Delta Blues role confirmed; Vicksburg assignment NOT independently verified.</t>
+        </is>
+      </c>
+      <c r="L25" s="54" t="n"/>
+      <c r="M25" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -45881,6 +46504,19 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I26" s="54" t="n"/>
+      <c r="J26" s="54" t="n"/>
+      <c r="K26" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L26" s="54" t="n"/>
+      <c r="M26" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="54" t="inlineStr">
@@ -45919,6 +46555,31 @@
           <t>News quote</t>
         </is>
       </c>
+      <c r="I27" s="54" t="inlineStr">
+        <is>
+          <t>drunyan@invenergy.com</t>
+        </is>
+      </c>
+      <c r="J27" s="54" t="inlineStr">
+        <is>
+          <t>+1 281-831-9568</t>
+        </is>
+      </c>
+      <c r="K27" s="54" t="inlineStr">
+        <is>
+          <t>Published Invenergy business contact; Sycamore-specific buying authority unconfirmed.</t>
+        </is>
+      </c>
+      <c r="L27" s="56" t="inlineStr">
+        <is>
+          <t>https://apps.dnr.wi.gov/warp_ext/am_permittracking2.aspx?id=38822</t>
+        </is>
+      </c>
+      <c r="M27" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="54" t="inlineStr">
@@ -45957,6 +46618,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I28" s="54" t="n"/>
+      <c r="J28" s="54" t="n"/>
+      <c r="K28" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L28" s="54" t="n"/>
+      <c r="M28" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="54" t="inlineStr">
@@ -45995,6 +46669,19 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I29" s="54" t="n"/>
+      <c r="J29" s="54" t="n"/>
+      <c r="K29" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L29" s="54" t="n"/>
+      <c r="M29" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="54" t="inlineStr">
@@ -46033,6 +46720,19 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I30" s="54" t="n"/>
+      <c r="J30" s="54" t="n"/>
+      <c r="K30" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L30" s="54" t="n"/>
+      <c r="M30" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="54" t="inlineStr">
@@ -46071,6 +46771,19 @@
           <t>Company website</t>
         </is>
       </c>
+      <c r="I31" s="54" t="n"/>
+      <c r="J31" s="54" t="n"/>
+      <c r="K31" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L31" s="54" t="n"/>
+      <c r="M31" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="54" t="inlineStr">
@@ -46109,6 +46822,27 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I32" s="54" t="inlineStr">
+        <is>
+          <t>npress1@entergy.com</t>
+        </is>
+      </c>
+      <c r="J32" s="54" t="n"/>
+      <c r="K32" s="54" t="inlineStr">
+        <is>
+          <t>Historical business email: 2022 DOE report; reconfirm before use. Direct phone not found.</t>
+        </is>
+      </c>
+      <c r="L32" s="56" t="inlineStr">
+        <is>
+          <t>https://www.osti.gov/servlets/purl/1884860</t>
+        </is>
+      </c>
+      <c r="M32" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="54" t="inlineStr">
@@ -46147,6 +46881,19 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I33" s="54" t="n"/>
+      <c r="J33" s="54" t="n"/>
+      <c r="K33" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L33" s="54" t="n"/>
+      <c r="M33" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="54" t="inlineStr">
@@ -46185,6 +46932,19 @@
           <t>Org website</t>
         </is>
       </c>
+      <c r="I34" s="54" t="n"/>
+      <c r="J34" s="54" t="n"/>
+      <c r="K34" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L34" s="54" t="n"/>
+      <c r="M34" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="54" t="inlineStr">
@@ -46223,6 +46983,19 @@
           <t>Official website</t>
         </is>
       </c>
+      <c r="I35" s="54" t="n"/>
+      <c r="J35" s="54" t="n"/>
+      <c r="K35" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L35" s="54" t="n"/>
+      <c r="M35" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="54" t="inlineStr">
@@ -46265,6 +47038,23 @@
           <t>Official release</t>
         </is>
       </c>
+      <c r="I36" s="54" t="n"/>
+      <c r="J36" s="54" t="inlineStr">
+        <is>
+          <t>+1 504-576-4132</t>
+        </is>
+      </c>
+      <c r="K36" s="54" t="inlineStr">
+        <is>
+          <t>Media contact only; not procurement. Published media phone confirmed; original email not independently reconfirmed.</t>
+        </is>
+      </c>
+      <c r="L36" s="54" t="n"/>
+      <c r="M36" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
@@ -46303,6 +47093,27 @@
           <t>Regulatory filing</t>
         </is>
       </c>
+      <c r="I37" s="54" t="inlineStr">
+        <is>
+          <t>npress1@entergy.com</t>
+        </is>
+      </c>
+      <c r="J37" s="54" t="n"/>
+      <c r="K37" s="54" t="inlineStr">
+        <is>
+          <t>Historical business email: 2022 DOE report; reconfirm before use. Direct phone not found.</t>
+        </is>
+      </c>
+      <c r="L37" s="56" t="inlineStr">
+        <is>
+          <t>https://www.osti.gov/servlets/purl/1884860</t>
+        </is>
+      </c>
+      <c r="M37" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="54" t="inlineStr">
@@ -46341,6 +47152,19 @@
           <t>Secondary source - verify</t>
         </is>
       </c>
+      <c r="I38" s="54" t="n"/>
+      <c r="J38" s="54" t="n"/>
+      <c r="K38" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L38" s="54" t="n"/>
+      <c r="M38" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="54" t="inlineStr">
@@ -46381,48 +47205,884 @@
       <c r="H39" s="54" t="inlineStr">
         <is>
           <t>Company website / customs record</t>
+        </is>
+      </c>
+      <c r="I39" s="54" t="n"/>
+      <c r="J39" s="54" t="n"/>
+      <c r="K39" s="54" t="inlineStr">
+        <is>
+          <t>Original lead suggestion; assignment/contact details not independently confirmed in this review.</t>
+        </is>
+      </c>
+      <c r="L39" s="54" t="n"/>
+      <c r="M39" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside</t>
+        </is>
+      </c>
+      <c r="B40" s="54" t="inlineStr">
+        <is>
+          <t>Sycamore project team</t>
+        </is>
+      </c>
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t>Shared business route</t>
+        </is>
+      </c>
+      <c r="D40" s="54" t="inlineStr">
+        <is>
+          <t>Invenergy</t>
+        </is>
+      </c>
+      <c r="E40" s="54" t="inlineStr">
+        <is>
+          <t>Shared project contact</t>
+        </is>
+      </c>
+      <c r="F40" s="54" t="inlineStr">
+        <is>
+          <t>SycamoreRiverside@invenergy.com; +1 800-341-2319</t>
+        </is>
+      </c>
+      <c r="G40" s="56" t="inlineStr">
+        <is>
+          <t>https://sycamoreriverside.invenergy.com/contact-us</t>
+        </is>
+      </c>
+      <c r="H40" s="54" t="inlineStr">
+        <is>
+          <t>Shared project contact</t>
+        </is>
+      </c>
+      <c r="I40" s="54" t="inlineStr">
+        <is>
+          <t>SycamoreRiverside@invenergy.com</t>
+        </is>
+      </c>
+      <c r="J40" s="54" t="inlineStr">
+        <is>
+          <t>+1 800-341-2319</t>
+        </is>
+      </c>
+      <c r="K40" s="54" t="inlineStr">
+        <is>
+          <t>Shared project contact</t>
+        </is>
+      </c>
+      <c r="L40" s="56" t="inlineStr">
+        <is>
+          <t>https://sycamoreriverside.invenergy.com/contact-us</t>
+        </is>
+      </c>
+      <c r="M40" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="54" t="inlineStr">
+        <is>
+          <t>Vast Sands / Permian Basin</t>
+        </is>
+      </c>
+      <c r="B41" s="54" t="inlineStr">
+        <is>
+          <t>Supply chain routing</t>
+        </is>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t>Shared business route</t>
+        </is>
+      </c>
+      <c r="D41" s="54" t="inlineStr">
+        <is>
+          <t>Vistra</t>
+        </is>
+      </c>
+      <c r="E41" s="54" t="inlineStr">
+        <is>
+          <t>Email: supply chain; phone: supplier diversity. Not CEO direct contact</t>
+        </is>
+      </c>
+      <c r="F41" s="54" t="inlineStr">
+        <is>
+          <t>SupplyChain@Vistracorp.com; +1 214-812-8000</t>
+        </is>
+      </c>
+      <c r="G41" s="56" t="inlineStr">
+        <is>
+          <t>https://vistracorp.com/supply-chain/how-do-we-source/ | https://vistracorp.com/supply-chain/faq/</t>
+        </is>
+      </c>
+      <c r="H41" s="54" t="inlineStr">
+        <is>
+          <t>Email: supply chain; phone: supplier diversity. Not CEO direct contact</t>
+        </is>
+      </c>
+      <c r="I41" s="54" t="inlineStr">
+        <is>
+          <t>SupplyChain@Vistracorp.com</t>
+        </is>
+      </c>
+      <c r="J41" s="54" t="inlineStr">
+        <is>
+          <t>+1 214-812-8000</t>
+        </is>
+      </c>
+      <c r="K41" s="54" t="inlineStr">
+        <is>
+          <t>Email: supply chain; phone: supplier diversity. Not CEO direct contact</t>
+        </is>
+      </c>
+      <c r="L41" s="56" t="inlineStr">
+        <is>
+          <t>https://vistracorp.com/supply-chain/how-do-we-source/ | https://vistracorp.com/supply-chain/faq/</t>
+        </is>
+      </c>
+      <c r="M41" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId46"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Stephan Hardt | Power Generation — Verification • 29 October 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>11 records reviewed • 9 have a published email + phone route (direct, shared project or supplier support); 2 still need a suitable contact pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Publication checks only; no calls or emails sent. Exact unsupported commissioning dates cleared. Close dates, cable values and buying windows remain sales assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="53" t="n"/>
+      <c r="B4" s="53" t="n"/>
+      <c r="C4" s="53" t="n"/>
+      <c r="D4" s="53" t="n"/>
+      <c r="E4" s="53" t="n"/>
+      <c r="F4" s="53" t="n"/>
+      <c r="G4" s="53" t="n"/>
+      <c r="H4" s="53" t="n"/>
+      <c r="I4" s="53" t="n"/>
+      <c r="J4" s="53" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B5" s="54" t="inlineStr">
+        <is>
+          <t>Verified status</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>Timing / precision</t>
+        </is>
+      </c>
+      <c r="D5" s="54" t="inlineStr">
+        <is>
+          <t>Capacity reconciliation</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>Facts checked</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>Required follow-up</t>
+        </is>
+      </c>
+      <c r="G5" s="54" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="H5" s="54" t="inlineStr">
+        <is>
+          <t>Contact route</t>
+        </is>
+      </c>
+      <c r="I5" s="54" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="J5" s="54" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>Forest Junction Energy Center</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>Proposed / permitting</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>2031 target; no exact day confirmed</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>1203 MW retained; unit figure needs permit/EIA confirmation. Developer publishes 1.9 GW for Forest Junction + Union Depot together.</t>
+        </is>
+      </c>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t>Invenergy proposes gas generation in Calumet County, Wisconsin. Developer timeline shows development 2025–2027, construction 2028–2031 and operation in 2031.</t>
+        </is>
+      </c>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t>Confirm selected site, CPCN status, individual capacity, turbine count and transmission scope.</t>
+        </is>
+      </c>
+      <c r="G6" s="55" t="inlineStr">
+        <is>
+          <t>https://forestjunctionenergycenter.invenergy.com/news-and-resources</t>
+        </is>
+      </c>
+      <c r="H6" s="54" t="inlineStr">
+        <is>
+          <t>Daniel Birmingham — published business contact; Wisconsin DNR listing is for another Invenergy project</t>
+        </is>
+      </c>
+      <c r="I6" s="54" t="inlineStr">
+        <is>
+          <t>dbirmingham@invenergy.com</t>
+        </is>
+      </c>
+      <c r="J6" s="54" t="inlineStr">
+        <is>
+          <t>+1 312-582-1094</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t>Orange County Advanced Power Station (OCAPS)</t>
+        </is>
+      </c>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>2026-10-14 actual</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
+        <is>
+          <t>1215 MW confirmed</t>
+        </is>
+      </c>
+      <c r="E7" s="54" t="inlineStr">
+        <is>
+          <t>Entergy Texas placed the 1,215 MW combined-cycle OCAPS facility in service on October 14, 2026.</t>
+        </is>
+      </c>
+      <c r="F7" s="54" t="inlineStr">
+        <is>
+          <t>Treat remaining sales as separately qualified maintenance/spares work; whole-plant cable estimate is not an open order.</t>
+        </is>
+      </c>
+      <c r="G7" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-texas-orange-county-advanced-power-station-begins-delivering-reliable-power-to-southeast-texas</t>
+        </is>
+      </c>
+      <c r="H7" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I7" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J7" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>Vast Sands Power I (Vistra Permian Basin expansion)</t>
+        </is>
+      </c>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>FID announced; execution status to confirm</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>2028 input target; exact unit date unverified</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>440 MW retained for unit I; owner confirms 860 MW for two new units combined. Do not sum two 440 MW estimates as the published total.</t>
+        </is>
+      </c>
+      <c r="E8" s="54" t="inlineStr">
+        <is>
+          <t>Vistra announced final investment decision September 29, 2025 for two new Permian Basin gas units totaling 860 MW, expanding the site from 325 to 1,185 MW.</t>
+        </is>
+      </c>
+      <c r="F8" s="54" t="inlineStr">
+        <is>
+          <t>Resolve Vast Sands unit mapping, gross/net capacity and current construction/COD with developer.</t>
+        </is>
+      </c>
+      <c r="G8" s="55" t="inlineStr">
+        <is>
+          <t>https://hub.vistracorp.com/vistra-announces-plans-to-build-new-dispatchable-generation-in-texas/</t>
+        </is>
+      </c>
+      <c r="H8" s="54" t="inlineStr">
+        <is>
+          <t>Vistra supply chain email / supplier-diversity phone — shared routing, not Jim Burke</t>
+        </is>
+      </c>
+      <c r="I8" s="54" t="inlineStr">
+        <is>
+          <t>SupplyChain@Vistracorp.com</t>
+        </is>
+      </c>
+      <c r="J8" s="54" t="inlineStr">
+        <is>
+          <t>+1 214-812-8000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>Plant Yates Unit 9 (Yates CT Units 8-10)</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>Under construction per owner update</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>By end 2027 for all 3 units; Unit 9 day unverified</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>482.8 MW retained as input nameplate; owner release reports approximately 1300 MW across 3 units. Basis needs reconciliation.</t>
+        </is>
+      </c>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t>Georgia Power confirms Unit 9 turbine/generator delivery in December 2025. Units 8–10 use Mitsubishi M501JAC simple-cycle turbines.</t>
+        </is>
+      </c>
+      <c r="F9" s="54" t="inlineStr">
+        <is>
+          <t>Confirm Unit 9 commissioning date and nameplate versus operating capacity; do not assume cable purchase status.</t>
+        </is>
+      </c>
+      <c r="G9" s="55" t="inlineStr">
+        <is>
+          <t>https://www.georgiapower.com/news-hub/press-releases/turbine-generator-unit-9-plant-yates.html</t>
+        </is>
+      </c>
+      <c r="H9" s="54" t="inlineStr">
+        <is>
+          <t>Not found — action required</t>
+        </is>
+      </c>
+      <c r="I9" s="54" t="n"/>
+      <c r="J9" s="54" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Ironwood Power Station</t>
+        </is>
+      </c>
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>Groundbreaking confirmed</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>2028 owner planning target</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>446 MW owner figure; EPC page rounds to 400 MW</t>
+        </is>
+      </c>
+      <c r="E10" s="54" t="inlineStr">
+        <is>
+          <t>Entergy Arkansas broke ground August 20, 2026 on Ironwood, a 446 MW simple-cycle plant at the existing Lake Catherine site.</t>
+        </is>
+      </c>
+      <c r="F10" s="54" t="inlineStr">
+        <is>
+          <t>Request project procurement contact and remaining electrical packages through the TSL vendor route.</t>
+        </is>
+      </c>
+      <c r="G10" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-arkansas-breaks-ground-on-ironwood-power-station</t>
+        </is>
+      </c>
+      <c r="H10" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I10" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J10" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>Person County Combined Cycle 1 (CC1)</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>EPC awarded; construction planned/underway</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>2028 target; exact quarter/day unverified</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>1360 MW confirmed</t>
+        </is>
+      </c>
+      <c r="E11" s="54" t="inlineStr">
+        <is>
+          <t>Zachry announced the EPC award August 6, 2025 for Duke Energy’s 1,360 MW, 2x1 Person County CC1 at Roxboro.</t>
+        </is>
+      </c>
+      <c r="F11" s="54" t="inlineStr">
+        <is>
+          <t>Use Zachry procurement registration; named buyer email/phone still required. Confirm current bid schedule.</t>
+        </is>
+      </c>
+      <c r="G11" s="55" t="inlineStr">
+        <is>
+          <t>https://zachrygroup.com/press-releases/Duke_Energy_Awards_EPC_Contract_for_the_first_Person_County_Combined_Cycle_Project_to_Zachry_Group.html</t>
+        </is>
+      </c>
+      <c r="H11" s="54" t="inlineStr">
+        <is>
+          <t>Not found — action required</t>
+        </is>
+      </c>
+      <c r="I11" s="54" t="n"/>
+      <c r="J11" s="54" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
+          <t>Delta Blues Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>Construction confirmed</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>2028 target; exact month/day unverified</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>754 MW confirmed</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t>Entergy’s May 19, 2026 update confirms HRSG erection and combustion-turbine delivery at Delta Blues in Greenville. Ernest Rufus is identified as senior manager, capital projects.</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t>DONE: 1950s Andrus claim removed. Note: construction milestones do not prove cable packages are already purchased.</t>
+        </is>
+      </c>
+      <c r="G12" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/blog/delta-blues-reaches-important-milestone-in-construction</t>
+        </is>
+      </c>
+      <c r="H12" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I12" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J12" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="54" t="inlineStr">
+        <is>
+          <t>Vicksburg Advanced Power Station</t>
+        </is>
+      </c>
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>Construction project</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>August 2028 expected completion; no exact day</t>
+        </is>
+      </c>
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>754 MW confirmed</t>
+        </is>
+      </c>
+      <c r="E13" s="54" t="inlineStr">
+        <is>
+          <t>Entergy plans Vicksburg Advanced Power Station at the former Baxter Wilson site in Warren County. Baxter Wilson retired in 2022.</t>
+        </is>
+      </c>
+      <c r="F13" s="54" t="inlineStr">
+        <is>
+          <t>Confirm Ernest Rufus covers Vicksburg (Delta Blues role confirmed only); request named project buyer.</t>
+        </is>
+      </c>
+      <c r="G13" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergymississippi.com/generation/vicksburg</t>
+        </is>
+      </c>
+      <c r="H13" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I13" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J13" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>Sycamore Riverside Energy Center</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>Proposed acquisition; regulatory decision pending</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>March 2029 transfer target; subject to completion/approval</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>918 MW confirmed in acquisition announcement</t>
+        </is>
+      </c>
+      <c r="E14" s="54" t="inlineStr">
+        <is>
+          <t>I&amp;M announced a request to acquire Invenergy’s Sycamore Riverside facility on completion, subject to IURC approval.</t>
+        </is>
+      </c>
+      <c r="F14" s="54" t="inlineStr">
+        <is>
+          <t>Do not treat acquisition as approved or closed. Verify Niland’s current project assignment and procurement scope.</t>
+        </is>
+      </c>
+      <c r="G14" s="55" t="inlineStr">
+        <is>
+          <t>https://www.aep.com/news/stories/view/11850/</t>
+        </is>
+      </c>
+      <c r="H14" s="54" t="inlineStr">
+        <is>
+          <t>Sycamore project team — shared, not John Niland</t>
+        </is>
+      </c>
+      <c r="I14" s="54" t="inlineStr">
+        <is>
+          <t>SycamoreRiverside@invenergy.com</t>
+        </is>
+      </c>
+      <c r="J14" s="54" t="inlineStr">
+        <is>
+          <t>+1 800-341-2319</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>Franklin Farms Power Station (Units 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Groundbreaking confirmed</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>Late 2028 owner target</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>Changed 1500 rounded to 1508 MW planning/EPC total for two units</t>
+        </is>
+      </c>
+      <c r="E15" s="54" t="inlineStr">
+        <is>
+          <t>Entergy Louisiana broke ground December 1, 2025 on Franklin Farms in Richland Parish. Two combined-cycle units support system growth including Meta demand.</t>
+        </is>
+      </c>
+      <c r="F15" s="54" t="inlineStr">
+        <is>
+          <t>DONE: 1,508 MW used. Confirm land ownership and electrical package status.</t>
+        </is>
+      </c>
+      <c r="G15" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergy.com/news/entergy-louisiana-breaks-ground-on-new-state-of-the-art-generation-facilities-to-power-reliability-growth-and-innovation</t>
+        </is>
+      </c>
+      <c r="H15" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I15" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J15" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t>Waterford 5 Power Station</t>
+        </is>
+      </c>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>Site preparation; main construction scheduled</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>2029 owner target; June date not substantiated</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>Changed 820 input nameplate to 754 MW owner planning basis; reconcile gross/net before technical sizing</t>
+        </is>
+      </c>
+      <c r="E16" s="54" t="inlineStr">
+        <is>
+          <t>Owner locates Waterford 5 in Taft, St. Charles Parish. Site preparation began November 2025; construction is scheduled for late 2026 with completion in 2029.</t>
+        </is>
+      </c>
+      <c r="F16" s="54" t="inlineStr">
+        <is>
+          <t>Owner location takes precedence over conflicting EPC page label (Big Cajun/Jarreau). Waterford 6 remains a separate project.</t>
+        </is>
+      </c>
+      <c r="G16" s="55" t="inlineStr">
+        <is>
+          <t>https://www.entergylouisiana.com/waterford5-6</t>
+        </is>
+      </c>
+      <c r="H16" s="54" t="inlineStr">
+        <is>
+          <t>Entergy supplier support — shared, not named lead</t>
+        </is>
+      </c>
+      <c r="I16" s="54" t="inlineStr">
+        <is>
+          <t>esupplier@entergy.com</t>
+        </is>
+      </c>
+      <c r="J16" s="54" t="inlineStr">
+        <is>
+          <t>+1 844-387-9675</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Set award date within 12-24 months of COD and close date at COD + 6 months
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2018,9 +2018,11 @@
         <v>48213</v>
       </c>
       <c r="X7" s="45" t="n">
-        <v>47299</v>
-      </c>
-      <c r="Y7" s="46" t="n"/>
+        <v>48395</v>
+      </c>
+      <c r="Y7" s="45" t="n">
+        <v>47483</v>
+      </c>
       <c r="Z7" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2073,7 +2075,7 @@
       </c>
       <c r="AJ7" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030 (award date set to COD-24 mo). EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="AK7" s="38" t="inlineStr">
@@ -2196,9 +2198,11 @@
         <v>46309</v>
       </c>
       <c r="X8" s="45" t="n">
-        <v>46507</v>
-      </c>
-      <c r="Y8" s="46" t="n"/>
+        <v>46491</v>
+      </c>
+      <c r="Y8" s="45" t="n">
+        <v>45944</v>
+      </c>
       <c r="Z8" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2251,7 +2255,7 @@
       </c>
       <c r="AJ8" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). New-build award passed; aftermarket/MRO opportunity (first spring outage ~Apr 2027 - estimate, not sourced). Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="AK8" s="38" t="inlineStr">
@@ -2364,9 +2368,11 @@
         <v>46874</v>
       </c>
       <c r="X9" s="45" t="n">
+        <v>47058</v>
+      </c>
+      <c r="Y9" s="45" t="n">
         <v>46418</v>
       </c>
-      <c r="Y9" s="46" t="n"/>
       <c r="Z9" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2419,7 +2425,7 @@
       </c>
       <c r="AJ9" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="AK9" s="38" t="inlineStr">
@@ -2532,9 +2538,11 @@
         <v>46568</v>
       </c>
       <c r="X10" s="45" t="n">
-        <v>46371</v>
-      </c>
-      <c r="Y10" s="46" t="n"/>
+        <v>46751</v>
+      </c>
+      <c r="Y10" s="45" t="n">
+        <v>46203</v>
+      </c>
       <c r="Z10" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2587,7 +2595,7 @@
       </c>
       <c r="AJ10" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium (award date set to COD-12 mo; already passed). Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="AK10" s="38" t="inlineStr">
@@ -2700,9 +2708,11 @@
         <v>47118</v>
       </c>
       <c r="X11" s="45" t="n">
+        <v>47299</v>
+      </c>
+      <c r="Y11" s="45" t="n">
         <v>46477</v>
       </c>
-      <c r="Y11" s="46" t="n"/>
       <c r="Z11" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2755,7 +2765,7 @@
       </c>
       <c r="AJ11" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="AK11" s="38" t="inlineStr">
@@ -2868,9 +2878,11 @@
         <v>47118</v>
       </c>
       <c r="X12" s="45" t="n">
+        <v>47299</v>
+      </c>
+      <c r="Y12" s="45" t="n">
         <v>46416</v>
       </c>
-      <c r="Y12" s="46" t="n"/>
       <c r="Z12" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -2923,7 +2935,7 @@
       </c>
       <c r="AJ12" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="AK12" s="38" t="inlineStr">
@@ -3044,9 +3056,11 @@
         <v>46874</v>
       </c>
       <c r="X13" s="45" t="n">
+        <v>47058</v>
+      </c>
+      <c r="Y13" s="45" t="n">
         <v>46356</v>
       </c>
-      <c r="Y13" s="46" t="n"/>
       <c r="Z13" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -3222,9 +3236,11 @@
         <v>46966</v>
       </c>
       <c r="X14" s="45" t="n">
+        <v>47150</v>
+      </c>
+      <c r="Y14" s="45" t="n">
         <v>46371</v>
       </c>
-      <c r="Y14" s="46" t="n"/>
       <c r="Z14" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -3392,9 +3408,11 @@
         <v>47208</v>
       </c>
       <c r="X15" s="45" t="n">
+        <v>47391</v>
+      </c>
+      <c r="Y15" s="45" t="n">
         <v>46568</v>
       </c>
-      <c r="Y15" s="46" t="n"/>
       <c r="Z15" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -3447,7 +3465,7 @@
       </c>
       <c r="AJ15" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="AK15" s="38" t="inlineStr">
@@ -3562,9 +3580,11 @@
         <v>47088</v>
       </c>
       <c r="X16" s="45" t="n">
+        <v>47270</v>
+      </c>
+      <c r="Y16" s="45" t="n">
         <v>46416</v>
       </c>
-      <c r="Y16" s="46" t="n"/>
       <c r="Z16" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -3617,7 +3637,7 @@
       </c>
       <c r="AJ16" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="AK16" s="38" t="inlineStr">
@@ -3732,9 +3752,11 @@
         <v>47270</v>
       </c>
       <c r="X17" s="45" t="n">
+        <v>47453</v>
+      </c>
+      <c r="Y17" s="45" t="n">
         <v>46660</v>
       </c>
-      <c r="Y17" s="46" t="n"/>
       <c r="Z17" s="37" t="inlineStr">
         <is>
           <t>Power Generation</t>
@@ -3787,7 +3809,7 @@
       </c>
       <c r="AJ17" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="AK17" s="38" t="inlineStr">
@@ -14882,7 +14904,7 @@
       <c r="CF7" s="39" t="n"/>
       <c r="CG7" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030. EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: CPCN filing expected fall 2026 (PSC docket 5-CE-162), construction start Q4 2027, COD Dec 2031 -&gt; BOP cable likely released in phases Q4 2028-Q2 2030 (award date set to COD-24 mo). EPC not named (Invenergy has used Kiewit elsewhere - unconfirmed). We Energies (Brendan Conway, spokesperson) may acquire; precedent: PSC approved Invenergy Red Oak Ridge/Foundry Ridge for We Energies Oct 15, 2026. Yes Energy shows 2030 COD; public sources Dec 2031.</t>
         </is>
       </c>
       <c r="CH7" s="38" t="inlineStr">
@@ -15175,7 +15197,7 @@
       <c r="CF8" s="39" t="n"/>
       <c r="CG8" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). Close date = estimated first spring maintenance outage (MRO/spares) - estimate, not sourced. Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
+          <t>*RPBD* In service Oct 14, 2026 - new-build window passed (~2023-24). New-build award passed; aftermarket/MRO opportunity (first spring outage ~Apr 2027 - estimate, not sourced). Other contacts: David Borde (CEO, Entergy Texas); James Malone (Dir. Business Development, Sargent &amp; Lundy).</t>
         </is>
       </c>
       <c r="CH8" s="38" t="inlineStr">
@@ -15464,7 +15486,7 @@
       <c r="CF9" s="39" t="n"/>
       <c r="CG9" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: FID Sep 2025; $583M TEF loan (Jun 2026) with $172M drawn by 6/30/26 = heavy early spend; COD May/Jun 2028 -&gt; cable window Dec 2026-Jun 2027, early packages may already be placed. EPC/OEM not public. No project-level contact public - Jim Burke is exec-level only (quoted in releases). TCEQ NAPD for permit 178462 should list applicant contact (Luminant Generation Co).</t>
         </is>
       </c>
       <c r="CH9" s="38" t="inlineStr">
@@ -15761,7 +15783,7 @@
       <c r="CF10" s="39" t="n"/>
       <c r="CG10" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium. Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
+          <t>*RPBD* LOW PROBABILITY: Unit 8 COD Q4 2026, Unit 9 Q2 2027, Unit 10 Q3 2027 (Southern Q2 2026 10-Q). Bulk cable likely bought 2024-25 by Mitsubishi/B&amp;V consortium (award date set to COD-12 mo; already passed). Remaining: Unit 10 top-ups, change orders, spares. Other contacts: Cheryl Boddiford (SVP Mfg &amp; Supply Chain, Mitsubishi Power); Rick Janik (B&amp;V PM on Plant Barry Unit 8 - same EPC pairing, not confirmed for Yates). GA PSC docket 55931.</t>
         </is>
       </c>
       <c r="CH10" s="38" t="inlineStr">
@@ -16054,7 +16076,7 @@
       <c r="CF11" s="39" t="n"/>
       <c r="CG11" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: site construction Q2 2026-Q2 2028, groundbreaking Aug 20 2026, COD Q4 2028 -&gt; bulk cable after underground/foundations ~Q1-Q2 2027. Best new-buy opportunity. TSL procures in its own name; S&amp;L writes cable specs/BOMs. TSL address: 8900 Renner Blvd, Lenexa KS 66219. Other contacts: Laura Landreaux (CEO, Entergy AR); Louise Duncan (VP Power Plant Ops, Entergy AR); Jason Rees (Dir. Procurement, Entergy - LinkedIn, verify). Entergy supplier registration: esupplier@entergy.com.</t>
         </is>
       </c>
       <c r="CH11" s="38" t="inlineStr">
@@ -16359,7 +16381,7 @@
       <c r="CF12" s="39" t="n"/>
       <c r="CG12" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: Zachry EPC Aug 2025, groundbreaking Feb 13 2026, first GE Vernova GT on site Jul 23 2026, Zachry craft hiring from Jul 2026; COD Q4 2028 (SC ORS) -&gt; bulk MV/600V/tray bid likely now; act immediately. CC2 (Q4 2029, likely Zachry) -&gt; separate close ~12/15/2027. Other contacts: Ralph Biediger (EPC Group President, Zachry); Bill Norton (Duke spokesperson). Utility is Duke Energy Progress (not DEC).</t>
         </is>
       </c>
       <c r="CH12" s="38" t="inlineStr">
@@ -17254,7 +17276,7 @@
       <c r="CF15" s="39" t="n"/>
       <c r="CG15" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: Boldt lists construction Sep 2026-Feb 2029 (built at risk before IURC order expected end-2026); COD Mar 31 2029 -&gt; cable window Q1-Q3 2027; Invenergy/Boldt buy, not I&amp;M. Other contacts: Daniel Runyan (SVP Development, Invenergy); Steve Baker (President &amp; COO, I&amp;M); Timothy B. Gaul (Dir. Regulated Infrastructure Development, AEPSC); Timothy C. Kerns (Sterling Industrial - owner's engineer witness). PJM (not MISO), 918 MW SC (not 1,150 MW CC).</t>
         </is>
       </c>
       <c r="CH15" s="38" t="inlineStr">
@@ -17549,7 +17571,7 @@
       <c r="CF16" s="39" t="n"/>
       <c r="CG16" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: groundbreaking Dec 1 2025, COD Dec 2028; IMI valve order Sep 2026 says detailed engineering still active -&gt; cable window Dec 2026-Jun 2027, early MV/grounding packages possibly Q4 2026. EPC TSL Power Partners/Kiewit + Mitsubishi. Other contacts: Phillip May (CEO, Entergy LA); Carlos Ruiz (VP Power Development, Entergy); Jim Niemiec (VP &amp; Chief Supply Chain Officer, Entergy); media Brandon Scardigli 504-576-4132. Separate 500 kV transmission opportunity.</t>
         </is>
       </c>
       <c r="CH16" s="38" t="inlineStr">
@@ -17854,7 +17876,7 @@
       <c r="CF17" s="39" t="n"/>
       <c r="CG17" s="38" t="inlineStr">
         <is>
-          <t>*RPBD* CLOSE DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
+          <t>*RPBD* AWARD (PO) DATE BASIS: site prep since Nov 2025, main construction late 2026, COD 2029 -&gt; cable window mid-2027-mid-2028. Waterford 6 (754 MW, ~Jul 2030, LPSC vote Dec 16 2026, same EPC) - pitch combined WF5+6 buy (~$3.75B program). Other contact: Michelle Berg (Entergy, parish council briefing - secondary source).</t>
         </is>
       </c>
       <c r="CH17" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Use Stage as sales stage: Open unless delayed or closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ne5CA7hEAcFrvqgbqau8k
</commit_message>
<xml_diff>
--- a/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
+++ b/Projects_and_Leads_Gas_Leads_2026-10-29.xlsx
@@ -2470,7 +2470,7 @@
       </c>
       <c r="C10" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D10" s="38" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D11" s="38" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="C12" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D12" s="38" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D13" s="38" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="C14" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D14" s="38" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="C16" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D16" s="38" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C18" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D18" s="38" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D21" s="38" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="C22" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D22" s="38" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="C24" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D24" s="38" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D25" s="38" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D26" s="38" t="inlineStr">

</xml_diff>